<commit_message>
feat: update PPV end-to-end automation, sort reports, and enhance HTML report generator
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -15,8 +15,7 @@
     <sheet name="Upgrade Confirmation page" sheetId="10" r:id="rId10"/>
     <sheet name="Phone Number page" sheetId="11" r:id="rId11"/>
     <sheet name="OTP page" sheetId="12" r:id="rId12"/>
-    <sheet name="Home of Boxing" sheetId="13" r:id="rId13"/>
-    <sheet name="Home page" sheetId="14" r:id="rId14"/>
+    <sheet name="Home page" sheetId="13" r:id="rId13"/>
   </sheets>
 </workbook>
 </file>
@@ -425,7 +424,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Don&amp;apos;t Miss Live on DAZN Section</v>
+        <v>Don't Miss Live on DAZN Section</v>
       </c>
       <c r="B2" t="str">
         <v>Yes</v>
@@ -472,7 +471,7 @@
         <v>Buy Now Button</v>
       </c>
       <c r="B6" t="str">
-        <v>Buy now</v>
+        <v>Yes</v>
       </c>
       <c r="C6" t="str">
         <v>landing</v>
@@ -732,7 +731,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:C22"/>
   </ignoredErrors>
@@ -792,7 +790,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
@@ -816,7 +813,7 @@
         <v>Page Title</v>
       </c>
       <c r="B2" t="str">
-        <v>Verify your phone</v>
+        <v>Enter the code below to continue</v>
       </c>
     </row>
     <row r="3">
@@ -852,7 +849,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
   </ignoredErrors>
@@ -861,7 +857,12 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C6"/>
+  <cols>
+    <col min="1" max="1" width="21.83203125" customWidth="1"/>
+    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -876,21 +877,21 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>home-boxing-banner</v>
+        <v>home-biggest-fights</v>
       </c>
       <c r="B2" t="str">
-        <v>Best of Boxing Section</v>
+        <v>The Biggest Fights Heading</v>
       </c>
       <c r="C2" t="str">
-        <v>Present</v>
+        <v>The Biggest Fights</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>home-boxing-banner</v>
+        <v>home-biggest-fights</v>
       </c>
       <c r="B3" t="str">
-        <v>Banner - Event Title</v>
+        <v>PPV Name</v>
       </c>
       <c r="C3" t="str">
         <v>{{PPV_NAME}}</v>
@@ -898,10 +899,10 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>home-boxing-banner</v>
+        <v>home-biggest-fights</v>
       </c>
       <c r="B4" t="str">
-        <v>Banner - Event Date</v>
+        <v>PPV Date and Time Text</v>
       </c>
       <c r="C4" t="str">
         <v>{{PPV_DATE}}</v>
@@ -909,268 +910,36 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>home-boxing-banner</v>
+        <v>home-biggest-fights</v>
       </c>
       <c r="B5" t="str">
-        <v>Banner - Event Description</v>
+        <v>PPV Image Present</v>
       </c>
       <c r="C5" t="str">
-        <v>{{PPV_DESCRIPTION}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>home-boxing-banner</v>
+        <v>home-biggest-fights</v>
       </c>
       <c r="B6" t="str">
-        <v>Banner - Buy Now CTA</v>
+        <v>Buy Now CTA</v>
       </c>
       <c r="C6" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>home-boxing-banner</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Banner - Fight Card CTA</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>home-boxing-tile</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Best of Boxing Section</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Present</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>home-boxing-tile</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Popup - Event Title</v>
-      </c>
-      <c r="C9" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>home-boxing-tile</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Popup - Event Date</v>
-      </c>
-      <c r="C10" t="str">
-        <v>{{PPV_DATE}}</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>home-boxing-tile</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Popup - Promoter</v>
-      </c>
-      <c r="C11" t="str">
-        <v>{{PPV_PROMOTER}}</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>home-boxing-tile</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Popup - Buy Now CTA</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>home-boxing-tile</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Popup - Event Description</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>home-boxing-tile</v>
-      </c>
-      <c r="B14" t="str">
-        <v>Popup - Close Button</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Flow</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Field</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Expected</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>home-page-banner</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Banner - Event Title</v>
-      </c>
-      <c r="C2" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>home-page-banner</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Banner - Event Date</v>
-      </c>
-      <c r="C3" t="str">
-        <v>{{PPV_DATE}}</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>home-page-banner</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Banner - Event Description</v>
-      </c>
-      <c r="C4" t="str">
-        <v>{{PPV_DESCRIPTION}}</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>home-page-banner</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Banner - Buy Now CTA</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>home-page-banner</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Banner - Fight Card CTA</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>home-page-dont-miss</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Popup - Event Title</v>
-      </c>
-      <c r="C7" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>home-page-dont-miss</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Popup - Event Date</v>
-      </c>
-      <c r="C8" t="str">
-        <v>{{PPV_DATE}}</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>home-page-dont-miss</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Popup - Promoter</v>
-      </c>
-      <c r="C9" t="str">
-        <v>{{PPV_PROMOTER}}</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>home-page-dont-miss</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Popup - Buy Now CTA</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Visible</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>home-page-dont-miss</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Popup - Event Description</v>
-      </c>
-      <c r="C11" t="str">
-        <v>{{PPV_DESCRIPTION}}</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>home-page-dont-miss</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Popup - Close Button</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Visible</v>
+        <v>Buy now</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C55"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1210,7 +979,7 @@
         <v>Event Subtitle</v>
       </c>
       <c r="B4" t="str">
-        <v>{{BOXING_BANNER_SUBTITLE}}</v>
+        <v>Main Event  AO Arena, Manchester  11:30 pm.</v>
       </c>
       <c r="C4" t="str">
         <v>boxing</v>
@@ -1273,76 +1042,76 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Bundle Section Present</v>
+        <v>Upcoming Big Fights Heading</v>
       </c>
       <c r="B10" t="str">
-        <v>Yes</v>
+        <v>Upcoming Big Fights</v>
       </c>
       <c r="C10" t="str">
-        <v>boxing-bundle</v>
+        <v>boxing-upcoming</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Bundle Section Title</v>
+        <v>PPV Name</v>
       </c>
       <c r="B11" t="str">
-        <v>{{BUNDLE_SECTION_TITLE}}</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="C11" t="str">
-        <v>boxing-bundle</v>
+        <v>boxing-upcoming</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Bundle Section Subtitle</v>
+        <v>PPV Date and Time Text</v>
       </c>
       <c r="B12" t="str">
-        <v>{{BUNDLE_SECTION_SUBTITLE}}</v>
+        <v>{{PPV_DATE}}</v>
       </c>
       <c r="C12" t="str">
-        <v>boxing-bundle</v>
+        <v>boxing-upcoming</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Bundle Title</v>
+        <v>PPV Description Text</v>
       </c>
       <c r="B13" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>{{PPV_LOCATION}}</v>
       </c>
       <c r="C13" t="str">
-        <v>boxing-bundle</v>
+        <v>boxing-upcoming</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Bundle Description</v>
+        <v>PPV Image Present</v>
       </c>
       <c r="B14" t="str">
-        <v>{{BUNDLE_DESCRIPTION}}</v>
+        <v>Yes</v>
       </c>
       <c r="C14" t="str">
-        <v>boxing-bundle</v>
+        <v>boxing-upcoming</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Bundle Price</v>
+        <v>Buy Now CTA</v>
       </c>
       <c r="B15" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>Buy now</v>
       </c>
       <c r="C15" t="str">
-        <v>boxing-bundle</v>
+        <v>boxing-upcoming</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Bundle Original Price</v>
+        <v>Bundle Section Present</v>
       </c>
       <c r="B16" t="str">
-        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
+        <v>Yes</v>
       </c>
       <c r="C16" t="str">
         <v>boxing-bundle</v>
@@ -1350,10 +1119,10 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Bundle Save Badge</v>
+        <v>Bundle Section Title</v>
       </c>
       <c r="B17" t="str">
-        <v>{{BUNDLE_SAVE_BADGE}}</v>
+        <v>{{BUNDLE_SECTION_TITLE}}</v>
       </c>
       <c r="C17" t="str">
         <v>boxing-bundle</v>
@@ -1361,10 +1130,10 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Bundle Fight Count</v>
+        <v>Bundle Section Subtitle</v>
       </c>
       <c r="B18" t="str">
-        <v>{{BUNDLE_FIGHT_COUNT}}</v>
+        <v>{{BUNDLE_SECTION_SUBTITLE}}</v>
       </c>
       <c r="C18" t="str">
         <v>boxing-bundle</v>
@@ -1372,10 +1141,10 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Bundle PPV 1 Name</v>
+        <v>Bundle Title</v>
       </c>
       <c r="B19" t="str">
-        <v>{{BUNDLE_PPV1_NAME}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="C19" t="str">
         <v>boxing-bundle</v>
@@ -1383,10 +1152,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Bundle PPV 1 Date</v>
+        <v>Bundle Description</v>
       </c>
       <c r="B20" t="str">
-        <v>{{BUNDLE_PPV1_LANDING_DATE}}</v>
+        <v>{{BUNDLE_DESCRIPTION}}</v>
       </c>
       <c r="C20" t="str">
         <v>boxing-bundle</v>
@@ -1394,10 +1163,10 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Bundle PPV 1 Image</v>
+        <v>Bundle Price</v>
       </c>
       <c r="B21" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="C21" t="str">
         <v>boxing-bundle</v>
@@ -1405,10 +1174,10 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Bundle PPV 2 Name</v>
+        <v>Bundle Original Price</v>
       </c>
       <c r="B22" t="str">
-        <v>{{BUNDLE_PPV2_NAME}}</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="C22" t="str">
         <v>boxing-bundle</v>
@@ -1416,10 +1185,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Bundle PPV 2 Date</v>
+        <v>Bundle Save Badge</v>
       </c>
       <c r="B23" t="str">
-        <v>{{BUNDLE_PPV2_LANDING_DATE}}</v>
+        <v>{{BUNDLE_SAVE_BADGE}}</v>
       </c>
       <c r="C23" t="str">
         <v>boxing-bundle</v>
@@ -1427,10 +1196,10 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Bundle PPV 2 Image</v>
+        <v>Bundle Fight Count</v>
       </c>
       <c r="B24" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_FIGHT_COUNT}}</v>
       </c>
       <c r="C24" t="str">
         <v>boxing-bundle</v>
@@ -1438,10 +1207,10 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Get Started CTA</v>
+        <v>Bundle PPV 1 Name</v>
       </c>
       <c r="B25" t="str">
-        <v>Get Started</v>
+        <v>{{BUNDLE_PPV1_NAME}}</v>
       </c>
       <c r="C25" t="str">
         <v>boxing-bundle</v>
@@ -1449,76 +1218,76 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>Page Title</v>
+        <v>Bundle PPV 1 Date</v>
       </c>
       <c r="B26" t="str">
-        <v>Choose the right plan for you.</v>
+        <v>{{BUNDLE_PPV1_LANDING_DATE}}</v>
       </c>
       <c r="C26" t="str">
-        <v>boxing-bundle-ppv</v>
+        <v>boxing-bundle</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Header Sub Text</v>
+        <v>Bundle PPV 1 Image</v>
       </c>
       <c r="B27" t="str">
-        <v>To watch your pay-per-view, you&amp;apos;ll need a DAZN plan.</v>
+        <v>Yes</v>
       </c>
       <c r="C27" t="str">
-        <v>boxing-bundle-ppv</v>
+        <v>boxing-bundle</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Bundle Card Title</v>
+        <v>Bundle PPV 2 Name</v>
       </c>
       <c r="B28" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>{{BUNDLE_PPV2_NAME}}</v>
       </c>
       <c r="C28" t="str">
-        <v>boxing-bundle-ppv</v>
+        <v>boxing-bundle</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Bundle Card Description</v>
+        <v>Bundle PPV 2 Date</v>
       </c>
       <c r="B29" t="str">
-        <v>{{BUNDLE_PPV_CARD_DESCRIPTION}}</v>
+        <v>{{BUNDLE_PPV2_LANDING_DATE}}</v>
       </c>
       <c r="C29" t="str">
-        <v>boxing-bundle-ppv</v>
+        <v>boxing-bundle</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Bundle Card Selected</v>
+        <v>Bundle PPV 2 Image</v>
       </c>
       <c r="B30" t="str">
         <v>Yes</v>
       </c>
       <c r="C30" t="str">
-        <v>boxing-bundle-ppv</v>
+        <v>boxing-bundle</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Bundle Card Price</v>
+        <v>Get Started CTA</v>
       </c>
       <c r="B31" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>Get Started</v>
       </c>
       <c r="C31" t="str">
-        <v>boxing-bundle-ppv</v>
+        <v>boxing-bundle</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Bundle Card Original Price</v>
+        <v>Page Title</v>
       </c>
       <c r="B32" t="str">
-        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
+        <v>Choose the right plan for you.</v>
       </c>
       <c r="C32" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1526,10 +1295,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Bundle Card Save Badge</v>
+        <v>Header Sub Text</v>
       </c>
       <c r="B33" t="str">
-        <v>{{BUNDLE_SAVE_BADGE}}</v>
+        <v>To watch your pay-per-view, you'll need a DAZN plan.</v>
       </c>
       <c r="C33" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1537,10 +1306,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Bundle PPV 1 Full Name</v>
+        <v>Bundle Card Title</v>
       </c>
       <c r="B34" t="str">
-        <v>{{BUNDLE_PPV1_FULL_NAME}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="C34" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1548,10 +1317,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Bundle PPV 1 PPV Date</v>
+        <v>Bundle Card Description</v>
       </c>
       <c r="B35" t="str">
-        <v>{{BUNDLE_PPV1_DATE}}</v>
+        <v>{{BUNDLE_PPV_CARD_DESCRIPTION}}</v>
       </c>
       <c r="C35" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1559,7 +1328,7 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Bundle PPV 1 PPV Image</v>
+        <v>Bundle Card Selected</v>
       </c>
       <c r="B36" t="str">
         <v>Yes</v>
@@ -1570,10 +1339,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Bundle PPV 2 Full Name</v>
+        <v>Bundle Card Price</v>
       </c>
       <c r="B37" t="str">
-        <v>{{BUNDLE_PPV2_FULL_NAME}}</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="C37" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1581,10 +1350,10 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>Bundle PPV 2 PPV Date</v>
+        <v>Bundle Card Original Price</v>
       </c>
       <c r="B38" t="str">
-        <v>{{BUNDLE_PPV2_DATE}}</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="C38" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1592,10 +1361,10 @@
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>Bundle PPV 2 PPV Image</v>
+        <v>Bundle Card Save Badge</v>
       </c>
       <c r="B39" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_SAVE_BADGE}}</v>
       </c>
       <c r="C39" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1603,10 +1372,10 @@
     </row>
     <row r="40">
       <c r="A40" t="str">
-        <v>Upsell Section Present</v>
+        <v>Bundle PPV 1 Full Name</v>
       </c>
       <c r="B40" t="str">
-        <v>Yes</v>
+        <v>{{BUNDLE_PPV1_FULL_NAME}}</v>
       </c>
       <c r="C40" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1614,10 +1383,10 @@
     </row>
     <row r="41">
       <c r="A41" t="str">
-        <v>Upsell Badge</v>
+        <v>Bundle PPV 1 PPV Date</v>
       </c>
       <c r="B41" t="str">
-        <v>The Ultimate Fan Package</v>
+        <v>{{BUNDLE_PPV1_DATE}}</v>
       </c>
       <c r="C41" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1625,10 +1394,10 @@
     </row>
     <row r="42">
       <c r="A42" t="str">
-        <v>Upsell Plan Name</v>
+        <v>Bundle PPV 1 PPV Image</v>
       </c>
       <c r="B42" t="str">
-        <v>DAZN Ultimate</v>
+        <v>Yes</v>
       </c>
       <c r="C42" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1636,10 +1405,10 @@
     </row>
     <row r="43">
       <c r="A43" t="str">
-        <v>Upsell Price</v>
+        <v>Bundle PPV 2 Full Name</v>
       </c>
       <c r="B43" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
+        <v>{{BUNDLE_PPV2_FULL_NAME}}</v>
       </c>
       <c r="C43" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1647,10 +1416,10 @@
     </row>
     <row r="44">
       <c r="A44" t="str">
-        <v>Upsell Contract Text</v>
+        <v>Bundle PPV 2 PPV Date</v>
       </c>
       <c r="B44" t="str">
-        <v>Annual contract. Auto renews.</v>
+        <v>{{BUNDLE_PPV2_DATE}}</v>
       </c>
       <c r="C44" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1658,10 +1427,10 @@
     </row>
     <row r="45">
       <c r="A45" t="str">
-        <v>Fights Included Text</v>
+        <v>Bundle PPV 2 PPV Image</v>
       </c>
       <c r="B45" t="str">
-        <v>All these fights included and more.</v>
+        <v>Yes</v>
       </c>
       <c r="C45" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1669,10 +1438,10 @@
     </row>
     <row r="46">
       <c r="A46" t="str">
-        <v>Upsell Feature 1</v>
+        <v>Upsell Section Present</v>
       </c>
       <c r="B46" t="str">
-        <v>Minimum 12 pay-per-views a year included at no extra cost.</v>
+        <v>Yes</v>
       </c>
       <c r="C46" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1680,10 +1449,10 @@
     </row>
     <row r="47">
       <c r="A47" t="str">
-        <v>Upsell Feature 2</v>
+        <v>Upsell Badge</v>
       </c>
       <c r="B47" t="str">
-        <v>185+ fights a year from the world&amp;apos;s best promoters.</v>
+        <v>The Ultimate Fan Package</v>
       </c>
       <c r="C47" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1691,10 +1460,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Upsell Feature 3</v>
+        <v>Upsell Plan Name</v>
       </c>
       <c r="B48" t="str">
-        <v>HDR and Dolby 5.1 surround sound on select events</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="C48" t="str">
         <v>boxing-bundle-ppv</v>
@@ -1702,18 +1471,84 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>CTA Button</v>
+        <v>Upsell Price</v>
       </c>
       <c r="B49" t="str">
-        <v>Continue with DAZN Ultimate</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
       <c r="C49" t="str">
         <v>boxing-bundle-ppv</v>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Upsell Contract Text</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Annual contract. Auto renews.</v>
+      </c>
+      <c r="C50" t="str">
+        <v>boxing-bundle-ppv</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Fights Included Text</v>
+      </c>
+      <c r="B51" t="str">
+        <v>All these fights included and more.</v>
+      </c>
+      <c r="C51" t="str">
+        <v>boxing-bundle-ppv</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Upsell Feature 1</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Minimum 12 pay-per-views a year included at no extra cost.</v>
+      </c>
+      <c r="C52" t="str">
+        <v>boxing-bundle-ppv</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Upsell Feature 2</v>
+      </c>
+      <c r="B53" t="str">
+        <v>185+ fights a year from the world's best promoters.</v>
+      </c>
+      <c r="C53" t="str">
+        <v>boxing-bundle-ppv</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Upsell Feature 3</v>
+      </c>
+      <c r="B54" t="str">
+        <v>HDR and Dolby 5.1 surround sound on select events</v>
+      </c>
+      <c r="C54" t="str">
+        <v>boxing-bundle-ppv</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>CTA Button</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Continue with DAZN Ultimate</v>
+      </c>
+      <c r="C55" t="str">
+        <v>boxing-bundle-ppv</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C49"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C55"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1746,6 +1581,9 @@
       <c r="C2" t="str">
         <v>Choose the right plan for you.</v>
       </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -1755,7 +1593,10 @@
         <v>Header Sub Text</v>
       </c>
       <c r="C3" t="str">
-        <v>To watch your pay-per-view, you&amp;apos;ll need a DAZN plan.</v>
+        <v>To watch your pay-per-view, you'll need a DAZN plan.</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -1768,6 +1609,9 @@
       <c r="C4" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -1779,6 +1623,9 @@
       <c r="C5" t="str">
         <v>N/A</v>
       </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -1790,6 +1637,9 @@
       <c r="C6" t="str">
         <v>Yes</v>
       </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -1801,6 +1651,9 @@
       <c r="C7" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -1812,6 +1665,9 @@
       <c r="C8" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -1823,6 +1679,9 @@
       <c r="C9" t="str">
         <v>{{CURRENCY}}</v>
       </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -1848,6 +1707,9 @@
       <c r="C11" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -1859,6 +1721,9 @@
       <c r="C12" t="str">
         <v>Yes</v>
       </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -1870,6 +1735,9 @@
       <c r="C13" t="str">
         <v>{{PPV_DATE}}</v>
       </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -1881,6 +1749,9 @@
       <c r="C14" t="str">
         <v>Yes</v>
       </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -1892,6 +1763,9 @@
       <c r="C15" t="str">
         <v>PPV: {{PPV_NAME}}</v>
       </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -1903,6 +1777,9 @@
       <c r="C16" t="str">
         <v>{{PPV_CARD_DESCRIPTION}}</v>
       </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -1914,6 +1791,9 @@
       <c r="C17" t="str">
         <v>Yes</v>
       </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -1925,6 +1805,9 @@
       <c r="C18" t="str">
         <v>The Ultimate Fan Package</v>
       </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -1936,6 +1819,9 @@
       <c r="C19" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -1947,6 +1833,9 @@
       <c r="C20" t="str">
         <v>N/A</v>
       </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1958,6 +1847,9 @@
       <c r="C21" t="str">
         <v>{{UPSELL_PRICE}}</v>
       </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -1969,6 +1861,9 @@
       <c r="C22" t="str">
         <v>/month</v>
       </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -1980,6 +1875,9 @@
       <c r="C23" t="str">
         <v>N/A</v>
       </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -1991,6 +1889,9 @@
       <c r="C24" t="str">
         <v>{{UPSELL_OFFER_TEXT}}</v>
       </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -2002,6 +1903,9 @@
       <c r="C25" t="str">
         <v>{{UPSELL_SECTION_HEADING}}</v>
       </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -2013,6 +1917,9 @@
       <c r="C26" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -2024,6 +1931,9 @@
       <c r="C27" t="str">
         <v>Yes</v>
       </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -2035,6 +1945,9 @@
       <c r="C28" t="str">
         <v>{{PPV_DATE}}</v>
       </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -2046,6 +1959,9 @@
       <c r="C29" t="str">
         <v>N/A</v>
       </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -2057,6 +1973,9 @@
       <c r="C30" t="str">
         <v>N/A</v>
       </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -2068,6 +1987,9 @@
       <c r="C31" t="str">
         <v>N/A</v>
       </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -2079,6 +2001,9 @@
       <c r="C32" t="str">
         <v>N/A</v>
       </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -2090,6 +2015,9 @@
       <c r="C33" t="str">
         <v>N/A</v>
       </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -2101,6 +2029,9 @@
       <c r="C34" t="str">
         <v>{{UPSELL_FEATURE_1}}</v>
       </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -2112,6 +2043,9 @@
       <c r="C35" t="str">
         <v>N/A</v>
       </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -2123,6 +2057,9 @@
       <c r="C36" t="str">
         <v>{{UPSELL_FEATURE_2}}</v>
       </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -2134,6 +2071,9 @@
       <c r="C37" t="str">
         <v>{{UPSELL_FEATURE_3}}</v>
       </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -2145,6 +2085,9 @@
       <c r="C38" t="str">
         <v>N/A</v>
       </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -2156,6 +2099,9 @@
       <c r="C39" t="str">
         <v>N/A</v>
       </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -2167,6 +2113,9 @@
       <c r="C40" t="str">
         <v>N/A</v>
       </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -2178,6 +2127,9 @@
       <c r="C41" t="str">
         <v>N/A</v>
       </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -2189,6 +2141,9 @@
       <c r="C42" t="str">
         <v>{{PPV_CTA_TEXT}}</v>
       </c>
+      <c r="D42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -2214,6 +2169,9 @@
       <c r="C44" t="str">
         <v>Choose your plan</v>
       </c>
+      <c r="D44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -2225,6 +2183,9 @@
       <c r="C45" t="str">
         <v>Buy {{PPV_NAME}} with DAZN Standard or get it included in DAZN Ultimate.</v>
       </c>
+      <c r="D45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -2236,6 +2197,9 @@
       <c r="C46" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -2247,6 +2211,9 @@
       <c r="C47" t="str">
         <v>get it included in DAZN Ultimate.</v>
       </c>
+      <c r="D47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -2258,6 +2225,9 @@
       <c r="C48" t="str">
         <v>Yes</v>
       </c>
+      <c r="D48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -2269,6 +2239,9 @@
       <c r="C49" t="str">
         <v>{{PPV_DATE}}</v>
       </c>
+      <c r="D49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -2280,6 +2253,9 @@
       <c r="C50" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -2291,6 +2267,9 @@
       <c r="C51" t="str">
         <v>Yes</v>
       </c>
+      <c r="D51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -2302,6 +2281,9 @@
       <c r="C52" t="str">
         <v>Yes</v>
       </c>
+      <c r="D52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -2313,6 +2295,9 @@
       <c r="C53" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -2324,6 +2309,9 @@
       <c r="C54" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="D54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -2335,6 +2323,9 @@
       <c r="C55" t="str">
         <v>{{CURRENCY}}</v>
       </c>
+      <c r="D55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -2346,6 +2337,9 @@
       <c r="C56" t="str">
         <v>Choose your subscription</v>
       </c>
+      <c r="D56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -2357,6 +2351,9 @@
       <c r="C57" t="str">
         <v>Yes</v>
       </c>
+      <c r="D57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -2368,6 +2365,9 @@
       <c r="C58" t="str">
         <v>7-day free trial of DAZN Standard</v>
       </c>
+      <c r="D58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -2379,6 +2379,9 @@
       <c r="C59" t="str">
         <v>Yes</v>
       </c>
+      <c r="D59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -2390,6 +2393,9 @@
       <c r="C60" t="str">
         <v>Yes</v>
       </c>
+      <c r="D60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -2401,6 +2407,9 @@
       <c r="C61" t="str">
         <v>7-days free access to DAZN Standard.</v>
       </c>
+      <c r="D61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -2412,6 +2421,9 @@
       <c r="C62" t="str">
         <v>Cancel anytime during the trial and only pay for the fight. After the trial you move onto a Monthly Flex plan for {{CURRENCY}}{{MONTHLY_PRICE}}/month. You will not lose access to the pay-per-view[s].</v>
       </c>
+      <c r="D62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -2423,6 +2435,9 @@
       <c r="C63" t="str">
         <v>Yes</v>
       </c>
+      <c r="D63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -2434,6 +2449,9 @@
       <c r="C64" t="str">
         <v>Pay-per-views included</v>
       </c>
+      <c r="D64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -2445,6 +2463,9 @@
       <c r="C65" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="D65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -2456,6 +2477,9 @@
       <c r="C66" t="str">
         <v>From</v>
       </c>
+      <c r="D66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -2467,6 +2491,9 @@
       <c r="C67" t="str">
         <v>{{UPSELL_PRICE}}</v>
       </c>
+      <c r="D67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -2478,6 +2505,9 @@
       <c r="C68" t="str">
         <v>/ month</v>
       </c>
+      <c r="D68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -2489,6 +2519,9 @@
       <c r="C69" t="str">
         <v>Annual contract. Auto renews.</v>
       </c>
+      <c r="D69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -2500,6 +2533,9 @@
       <c r="C70" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -2511,6 +2547,9 @@
       <c r="C71" t="str">
         <v>Yes</v>
       </c>
+      <c r="D71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -2522,6 +2561,9 @@
       <c r="C72" t="str">
         <v>{{PPV_DATE}}</v>
       </c>
+      <c r="D72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -2533,6 +2575,9 @@
       <c r="C73" t="str">
         <v>Yes</v>
       </c>
+      <c r="D73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -2544,6 +2589,9 @@
       <c r="C74" t="str">
         <v>N/A</v>
       </c>
+      <c r="D74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -2555,6 +2603,9 @@
       <c r="C75" t="str">
         <v>N/A</v>
       </c>
+      <c r="D75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -2566,6 +2617,9 @@
       <c r="C76" t="str">
         <v>N/A</v>
       </c>
+      <c r="D76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -2577,6 +2631,9 @@
       <c r="C77" t="str">
         <v>N/A</v>
       </c>
+      <c r="D77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -2588,6 +2645,9 @@
       <c r="C78" t="str">
         <v>Pay-per-views included at no extra cost. Minimum of 12 events per year including {{PPV_NAME}}.</v>
       </c>
+      <c r="D78" t="str">
+        <v/>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -2599,6 +2659,9 @@
       <c r="C79" t="str">
         <v>{{PPV_NAME}}.</v>
       </c>
+      <c r="D79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -2610,6 +2673,9 @@
       <c r="C80" t="str">
         <v>HDR and Dolby 5.1 surround sound on select events.</v>
       </c>
+      <c r="D80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -2621,6 +2687,9 @@
       <c r="C81" t="str">
         <v>185+ fights a year from the best promoters</v>
       </c>
+      <c r="D81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -2632,6 +2701,9 @@
       <c r="C82" t="str">
         <v>Whats included</v>
       </c>
+      <c r="D82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -2643,6 +2715,9 @@
       <c r="C83" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="D83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -2654,6 +2729,9 @@
       <c r="C84" t="str">
         <v>get it included in DAZN Ultimate.</v>
       </c>
+      <c r="D84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -2665,6 +2743,9 @@
       <c r="C85" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="D85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -2676,6 +2757,9 @@
       <c r="C86" t="str">
         <v>Continue with PPV + 7-day free trial</v>
       </c>
+      <c r="D86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -2686,6 +2770,9 @@
       </c>
       <c r="C87" t="str">
         <v>N/A</v>
+      </c>
+      <c r="D87" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -2697,7 +2784,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:D37"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2709,6 +2796,9 @@
       <c r="C1" t="str">
         <v>Expected</v>
       </c>
+      <c r="D1" t="str">
+        <v>Flow</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -2720,6 +2810,9 @@
       <c r="C2" t="str">
         <v>{{PLAN_PAGE_TITLE}}</v>
       </c>
+      <c r="D2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -2731,6 +2824,9 @@
       <c r="C3" t="str">
         <v>Yes</v>
       </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -2742,6 +2838,9 @@
       <c r="C4" t="str">
         <v>Flex – Pay Monthly</v>
       </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -2753,6 +2852,9 @@
       <c r="C5" t="str">
         <v>{{FLEX_BADGE}}</v>
       </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -2764,6 +2866,9 @@
       <c r="C6" t="str">
         <v>{{FLEX_DESCRIPTION}}</v>
       </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -2775,6 +2880,9 @@
       <c r="C7" t="str">
         <v>Yes</v>
       </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -2786,6 +2894,9 @@
       <c r="C8" t="str">
         <v>{{FLEX_TODAY_TEXT}}</v>
       </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -2797,6 +2908,9 @@
       <c r="C9" t="str">
         <v>{{FLEX_FUTURE_TEXT}}</v>
       </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -2808,6 +2922,9 @@
       <c r="C10" t="str">
         <v>Yes</v>
       </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -2819,6 +2936,9 @@
       <c r="C11" t="str">
         <v>{{ANNUAL_SAVINGS_BADGE}}</v>
       </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -2830,6 +2950,9 @@
       <c r="C12" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -2841,6 +2964,9 @@
       <c r="C13" t="str">
         <v>1 MONTH FREE</v>
       </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -2852,6 +2978,9 @@
       <c r="C14" t="str">
         <v>then {{CURRENCY}}{{ANNUAL_PRICE}}/month for {{ANNUAL_MONTHS}} months</v>
       </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -2863,6 +2992,9 @@
       <c r="C15" t="str">
         <v>Annual contract. Auto renews.</v>
       </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -2872,7 +3004,10 @@
         <v>Annual Feature 1</v>
       </c>
       <c r="C16" t="str">
-        <v>185+ fights a year from the world&amp;apos;s best promoters.</v>
+        <v>185+ fights a year from the world's best promoters.</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -2885,6 +3020,9 @@
       <c r="C17" t="str">
         <v>Additional cost for pay-per-view events.</v>
       </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -2896,6 +3034,9 @@
       <c r="C18" t="str">
         <v>Full HD video resolution.</v>
       </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -2907,6 +3048,9 @@
       <c r="C19" t="str">
         <v>No</v>
       </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -2918,6 +3062,9 @@
       <c r="C20" t="str">
         <v>{{PLAN_CTA_BUTTON}}</v>
       </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -2929,6 +3076,9 @@
       <c r="C21" t="str">
         <v>{{PLAN_PAGE_TITLE}}</v>
       </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -2940,6 +3090,9 @@
       <c r="C22" t="str">
         <v>Yes</v>
       </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -2951,6 +3104,9 @@
       <c r="C23" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -2962,6 +3118,9 @@
       <c r="C24" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
+      <c r="D24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -2973,6 +3132,9 @@
       <c r="C25" t="str">
         <v>/ month</v>
       </c>
+      <c r="D25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -2984,6 +3146,9 @@
       <c r="C26" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
       </c>
+      <c r="D26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -2995,6 +3160,9 @@
       <c r="C27" t="str">
         <v>Yes</v>
       </c>
+      <c r="D27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -3006,6 +3174,9 @@
       <c r="C28" t="str">
         <v>Yes</v>
       </c>
+      <c r="D28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -3017,6 +3188,9 @@
       <c r="C29" t="str">
         <v>Annual - Pay Upfront</v>
       </c>
+      <c r="D29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -3028,6 +3202,9 @@
       <c r="C30" t="str">
         <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -3039,6 +3216,9 @@
       <c r="C31" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE_DISPLAY}}</v>
       </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -3050,6 +3230,9 @@
       <c r="C32" t="str">
         <v>/year</v>
       </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -3061,6 +3244,9 @@
       <c r="C33" t="str">
         <v>No</v>
       </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -3072,6 +3258,9 @@
       <c r="C34" t="str">
         <v>Minimum 12 pay-per-views a year included at no extra cost.</v>
       </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -3081,7 +3270,10 @@
         <v>Ultimate Feature 2</v>
       </c>
       <c r="C35" t="str">
-        <v>185+ fights a year from the world&amp;apos;s best promoters.</v>
+        <v>185+ fights a year from the world's best promoters.</v>
+      </c>
+      <c r="D35" t="str">
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -3094,6 +3286,9 @@
       <c r="C36" t="str">
         <v>HDR and Dolby 5.1 surround sound on select events.</v>
       </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -3105,17 +3300,20 @@
       <c r="C37" t="str">
         <v>{{PLAN_CTA_BUTTON}}</v>
       </c>
+      <c r="D37" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C37"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D37"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E98"/>
+  <dimension ref="A1:E96"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3145,7 +3343,10 @@
         <v>Header</v>
       </c>
       <c r="D2" t="str">
-        <v>Your payment is encrypted and you can change how you pay at any time.|81% OFF for your first month|20% OFF for 12 months|First month free</v>
+        <v>Your payment is encrypted and you can change how you pay at any time.</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -3161,6 +3362,9 @@
       <c r="D3" t="str">
         <v>Change</v>
       </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -3175,6 +3379,9 @@
       <c r="D4" t="str">
         <v>Yes</v>
       </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -3189,6 +3396,9 @@
       <c r="D5" t="str">
         <v>Yes</v>
       </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -3203,6 +3413,9 @@
       <c r="D6" t="str">
         <v>Yes</v>
       </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -3268,6 +3481,9 @@
       <c r="D10" t="str">
         <v>Yes</v>
       </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -3316,6 +3532,9 @@
       <c r="D13" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -3330,6 +3549,9 @@
       <c r="D14" t="str">
         <v>{{PAYMENT_PLAN_NAME}}</v>
       </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -3344,6 +3566,9 @@
       <c r="D15" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -3358,6 +3583,9 @@
       <c r="D16" t="str">
         <v>{{PAYMENT_FREE_TEXT}}</v>
       </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -3372,6 +3600,9 @@
       <c r="D17" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -3386,6 +3617,9 @@
       <c r="D18" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -3400,6 +3634,9 @@
       <c r="D19" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -3414,6 +3651,9 @@
       <c r="D20" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -3428,6 +3668,9 @@
       <c r="D21" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -3442,6 +3685,9 @@
       <c r="D22" t="str">
         <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -3456,6 +3702,9 @@
       <c r="D23" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -3470,6 +3719,9 @@
       <c r="D24" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -3484,6 +3736,9 @@
       <c r="D25" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -3498,6 +3753,9 @@
       <c r="D26" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="E26" t="str">
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -3512,6 +3770,9 @@
       <c r="D27" t="str">
         <v>{{RATE_PLAN_LABEL}}</v>
       </c>
+      <c r="E27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -3526,6 +3787,9 @@
       <c r="D28" t="str">
         <v>{{CURRENCY}}{{ANNUAL_PRICE}}</v>
       </c>
+      <c r="E28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -3540,6 +3804,9 @@
       <c r="D29" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E29" t="str">
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -3554,6 +3821,9 @@
       <c r="D30" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -3568,6 +3838,9 @@
       <c r="D31" t="str">
         <v>{{PPV_PRICE}}</v>
       </c>
+      <c r="E31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -3582,6 +3855,9 @@
       <c r="D32" t="str">
         <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
       </c>
+      <c r="E32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -3596,6 +3872,9 @@
       <c r="D33" t="str">
         <v>Yes</v>
       </c>
+      <c r="E33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -3610,6 +3889,9 @@
       <c r="D34" t="str">
         <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
+      <c r="E34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -3624,6 +3906,9 @@
       <c r="D35" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -3638,6 +3923,9 @@
       <c r="D36" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -3652,6 +3940,9 @@
       <c r="D37" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E37" t="str">
+        <v/>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
@@ -3666,6 +3957,9 @@
       <c r="D38" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -3678,7 +3972,10 @@
         <v>Rate Plan</v>
       </c>
       <c r="D39" t="str">
-        <v>{{PAYMENT_PLAN_LABEL}}</v>
+        <v>Annual - Pay Monthly</v>
+      </c>
+      <c r="E39" t="str">
+        <v/>
       </c>
     </row>
     <row r="40">
@@ -3694,6 +3991,9 @@
       <c r="D40" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
+      <c r="E40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -3708,6 +4008,9 @@
       <c r="D41" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -3722,6 +4025,9 @@
       <c r="D42" t="str">
         <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
+      <c r="E42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -3736,6 +4042,9 @@
       <c r="D43" t="str">
         <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -3750,6 +4059,9 @@
       <c r="D44" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -3764,6 +4076,9 @@
       <c r="D45" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -3778,6 +4093,9 @@
       <c r="D46" t="str">
         <v>Yes</v>
       </c>
+      <c r="E46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -3792,6 +4110,9 @@
       <c r="D47" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -3806,6 +4127,9 @@
       <c r="D48" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -3820,6 +4144,9 @@
       <c r="D49" t="str">
         <v>{{PPV_NAME}}</v>
       </c>
+      <c r="E49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -3834,6 +4161,9 @@
       <c r="D50" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E50" t="str">
+        <v/>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -3848,6 +4178,9 @@
       <c r="D51" t="str">
         <v>Annual - Pay Upfront</v>
       </c>
+      <c r="E51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -3862,6 +4195,9 @@
       <c r="D52" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
       </c>
+      <c r="E52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -3876,6 +4212,9 @@
       <c r="D53" t="str">
         <v>Today you pay</v>
       </c>
+      <c r="E53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -3890,6 +4229,9 @@
       <c r="D54" t="str">
         <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
+      <c r="E54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -3904,6 +4246,9 @@
       <c r="D55" t="str">
         <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E55" t="str">
+        <v/>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
@@ -3918,6 +4263,9 @@
       <c r="D56" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
+      <c r="E56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -3932,6 +4280,9 @@
       <c r="D57" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -3946,6 +4297,9 @@
       <c r="D58" t="str">
         <v>Yes</v>
       </c>
+      <c r="E58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -3960,6 +4314,9 @@
       <c r="D59" t="str">
         <v>{{PAYMENT_PAGE_TITLE}}</v>
       </c>
+      <c r="E59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -3974,6 +4331,9 @@
       <c r="D60" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -3988,6 +4348,9 @@
       <c r="D61" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E61" t="str">
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="str">
@@ -4002,6 +4365,9 @@
       <c r="D62" t="str">
         <v>{{BUNDLE_PRICE}}</v>
       </c>
+      <c r="E62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -4016,6 +4382,9 @@
       <c r="D63" t="str">
         <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
       </c>
+      <c r="E63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -4030,6 +4399,9 @@
       <c r="D64" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -4044,6 +4416,9 @@
       <c r="D65" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -4058,6 +4433,9 @@
       <c r="D66" t="str">
         <v>DAZN Standard</v>
       </c>
+      <c r="E66" t="str">
+        <v/>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -4072,6 +4450,9 @@
       <c r="D67" t="str">
         <v>Annual - Pay Monthly</v>
       </c>
+      <c r="E67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -4086,6 +4467,9 @@
       <c r="D68" t="str">
         <v>First month free</v>
       </c>
+      <c r="E68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -4100,6 +4484,9 @@
       <c r="D69" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -4114,6 +4501,9 @@
       <c r="D70" t="str">
         <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
+      <c r="E70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -4128,6 +4518,9 @@
       <c r="D71" t="str">
         <v>{{BUNDLE_PRICE}}</v>
       </c>
+      <c r="E71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -4142,6 +4535,9 @@
       <c r="D72" t="str">
         <v>{{BUNDLE_DISCOUNT}}</v>
       </c>
+      <c r="E72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -4156,6 +4552,9 @@
       <c r="D73" t="str">
         <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
       </c>
+      <c r="E73" t="str">
+        <v/>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -4170,6 +4569,9 @@
       <c r="D74" t="str">
         <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
       </c>
+      <c r="E74" t="str">
+        <v/>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -4184,6 +4586,9 @@
       <c r="D75" t="str">
         <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
+      <c r="E75" t="str">
+        <v/>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -4198,6 +4603,9 @@
       <c r="D76" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E76" t="str">
+        <v/>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -4212,6 +4620,9 @@
       <c r="D77" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E77" t="str">
+        <v/>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -4224,7 +4635,10 @@
         <v>Rate Plan</v>
       </c>
       <c r="D78" t="str">
-        <v>{{PAYMENT_PLAN_LABEL}}</v>
+        <v>Annual - Pay Monthly</v>
+      </c>
+      <c r="E78" t="str">
+        <v/>
       </c>
     </row>
     <row r="79">
@@ -4240,6 +4654,9 @@
       <c r="D79" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
+      <c r="E79" t="str">
+        <v/>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -4254,6 +4671,9 @@
       <c r="D80" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E80" t="str">
+        <v/>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -4268,6 +4688,9 @@
       <c r="D81" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E81" t="str">
+        <v/>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -4282,6 +4705,9 @@
       <c r="D82" t="str">
         <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
+      <c r="E82" t="str">
+        <v/>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -4296,6 +4722,9 @@
       <c r="D83" t="str">
         <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E83" t="str">
+        <v/>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -4310,6 +4739,9 @@
       <c r="D84" t="str">
         <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
+      <c r="E84" t="str">
+        <v/>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -4324,6 +4756,9 @@
       <c r="D85" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
+      <c r="E85" t="str">
+        <v/>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -4338,6 +4773,9 @@
       <c r="D86" t="str">
         <v>Choose how to pay</v>
       </c>
+      <c r="E86" t="str">
+        <v/>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -4352,6 +4790,9 @@
       <c r="D87" t="str">
         <v>DAZN Ultimate</v>
       </c>
+      <c r="E87" t="str">
+        <v/>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="str">
@@ -4366,6 +4807,9 @@
       <c r="D88" t="str">
         <v>Annual - Pay Upfront</v>
       </c>
+      <c r="E88" t="str">
+        <v/>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="str">
@@ -4380,6 +4824,9 @@
       <c r="D89" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
       </c>
+      <c r="E89" t="str">
+        <v/>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="str">
@@ -4394,6 +4841,9 @@
       <c r="D90" t="str">
         <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
+      <c r="E90" t="str">
+        <v/>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="str">
@@ -4408,6 +4858,9 @@
       <c r="D91" t="str">
         <v>{{BUNDLE_NAME}}</v>
       </c>
+      <c r="E91" t="str">
+        <v/>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="str">
@@ -4422,6 +4875,9 @@
       <c r="D92" t="str">
         <v>{{CURRENCY}}0</v>
       </c>
+      <c r="E92" t="str">
+        <v/>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -4436,6 +4892,9 @@
       <c r="D93" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
+      <c r="E93" t="str">
+        <v/>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -4450,6 +4909,9 @@
       <c r="D94" t="str">
         <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
+      <c r="E94" t="str">
+        <v/>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -4464,6 +4926,9 @@
       <c r="D95" t="str">
         <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
+      <c r="E95" t="str">
+        <v/>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -4478,39 +4943,13 @@
       <c r="D96" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="str">
-        <v>Ultimate</v>
-      </c>
-      <c r="B97" t="str">
-        <v>Annual Pay Monthly</v>
-      </c>
-      <c r="C97" t="str">
-        <v>Discount Badge</v>
-      </c>
-      <c r="D97" t="str">
-        <v>{{DISCOUNT_BADGE}}</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="str">
-        <v>Ultimate</v>
-      </c>
-      <c r="B98" t="str">
-        <v>Annual Pay Monthly Bundle</v>
-      </c>
-      <c r="C98" t="str">
-        <v>Discount Badge</v>
-      </c>
-      <c r="D98" t="str">
-        <v>{{DISCOUNT_BADGE}}</v>
+      <c r="E96" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E98"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E96"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4632,7 +5071,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B14"/>
   </ignoredErrors>
@@ -4708,7 +5146,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
   </ignoredErrors>
@@ -4904,7 +5341,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B23"/>
   </ignoredErrors>
@@ -5044,7 +5480,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:B16"/>
   </ignoredErrors>

</xml_diff>

<commit_message>
feat: configure Web PPV New User matrix workflow and add Figma design check script
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -15,7 +15,6 @@
     <sheet name="Upgrade Confirmation page" sheetId="10" r:id="rId10"/>
     <sheet name="Phone Number page" sheetId="11" r:id="rId11"/>
     <sheet name="OTP page" sheetId="12" r:id="rId12"/>
-    <sheet name="Home page" sheetId="13" r:id="rId13"/>
   </sheets>
 </workbook>
 </file>
@@ -855,88 +854,6 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
-  <cols>
-    <col min="1" max="1" width="21.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Flow</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Field</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Expected</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>home-biggest-fights</v>
-      </c>
-      <c r="B2" t="str">
-        <v>The Biggest Fights Heading</v>
-      </c>
-      <c r="C2" t="str">
-        <v>The Biggest Fights</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>home-biggest-fights</v>
-      </c>
-      <c r="B3" t="str">
-        <v>PPV Name</v>
-      </c>
-      <c r="C3" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>home-biggest-fights</v>
-      </c>
-      <c r="B4" t="str">
-        <v>PPV Date and Time Text</v>
-      </c>
-      <c r="C4" t="str">
-        <v>{{PPV_DATE}}</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>home-biggest-fights</v>
-      </c>
-      <c r="B5" t="str">
-        <v>PPV Image Present</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>home-biggest-fights</v>
-      </c>
-      <c r="B6" t="str">
-        <v>Buy Now CTA</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Buy now</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C55"/>
@@ -1873,7 +1790,7 @@
         <v>Upsell Billing Text</v>
       </c>
       <c r="C23" t="str">
-        <v>N/A</v>
+        <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
       </c>
       <c r="D23" t="str">
         <v/>
@@ -3313,7 +3230,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E96"/>
+  <dimension ref="A1:F100"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3331,6 +3248,9 @@
       <c r="E1" t="str">
         <v>Flow</v>
       </c>
+      <c r="F1" t="str">
+        <v>Type</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -3671,6 +3591,9 @@
       <c r="E21" t="str">
         <v/>
       </c>
+      <c r="F21" t="str">
+        <v>contains</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -3683,7 +3606,7 @@
         <v>Ultimate Upsell Text</v>
       </c>
       <c r="D22" t="str">
-        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
+        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -3858,6 +3781,9 @@
       <c r="E32" t="str">
         <v/>
       </c>
+      <c r="F32" t="str">
+        <v>contains</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -3887,7 +3813,7 @@
         <v>Ultimate Upsell Text</v>
       </c>
       <c r="D34" t="str">
-        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
+        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
       <c r="E34" t="str">
         <v/>
@@ -4079,6 +4005,9 @@
       <c r="E45" t="str">
         <v/>
       </c>
+      <c r="F45" t="str">
+        <v>contains</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -4283,6 +4212,9 @@
       <c r="E57" t="str">
         <v/>
       </c>
+      <c r="F57" t="str">
+        <v>contains</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -4402,6 +4334,9 @@
       <c r="E64" t="str">
         <v/>
       </c>
+      <c r="F64" t="str">
+        <v>contains</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -4572,6 +4507,9 @@
       <c r="E74" t="str">
         <v/>
       </c>
+      <c r="F74" t="str">
+        <v>contains</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -4584,7 +4522,7 @@
         <v>Ultimate Upsell Text</v>
       </c>
       <c r="D75" t="str">
-        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
+        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
       <c r="E75" t="str">
         <v/>
@@ -4759,6 +4697,9 @@
       <c r="E85" t="str">
         <v/>
       </c>
+      <c r="F85" t="str">
+        <v>contains</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -4946,10 +4887,75 @@
       <c r="E96" t="str">
         <v/>
       </c>
+      <c r="F96" t="str">
+        <v>contains</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="str">
+        <v>standard</v>
+      </c>
+      <c r="B97" t="str">
+        <v>monthly</v>
+      </c>
+      <c r="C97" t="str">
+        <v>Ultimate Upsell Banner Present</v>
+      </c>
+      <c r="D97" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="str">
+        <v>standard</v>
+      </c>
+      <c r="B98" t="str">
+        <v>monthly</v>
+      </c>
+      <c r="C98" t="str">
+        <v>Ultimate Upsell Price</v>
+      </c>
+      <c r="D98" t="str">
+        <v>{{ULTIMATE_ANNUAL_PAY_MONTHLY_PRICE}}</v>
+      </c>
+      <c r="F98" t="str">
+        <v>contains</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="str">
+        <v>standard</v>
+      </c>
+      <c r="B99" t="str">
+        <v>annual pay monthly</v>
+      </c>
+      <c r="C99" t="str">
+        <v>Ultimate Upsell Banner Present</v>
+      </c>
+      <c r="D99" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="str">
+        <v>standard</v>
+      </c>
+      <c r="B100" t="str">
+        <v>annual pay monthly</v>
+      </c>
+      <c r="C100" t="str">
+        <v>Ultimate Upsell Price</v>
+      </c>
+      <c r="D100" t="str">
+        <v>{{ULTIMATE_ANNUAL_PAY_MONTHLY_PRICE}}</v>
+      </c>
+      <c r="F100" t="str">
+        <v>contains</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E96"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F100"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5154,7 +5160,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:C23"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5163,6 +5169,9 @@
       <c r="B1" t="str">
         <v>Expected</v>
       </c>
+      <c r="C1" t="str">
+        <v>Type</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -5187,6 +5196,9 @@
       <c r="B4" t="str">
         <v>Buy {{PPV_NAME}}, or get it included in a DAZN Ultimate subscription</v>
       </c>
+      <c r="C4" t="str">
+        <v>contains</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -5299,6 +5311,9 @@
       <c r="B18" t="str">
         <v>{{UPSELL_FEATURE_1}}</v>
       </c>
+      <c r="C18" t="str">
+        <v>contains</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -5315,6 +5330,9 @@
       <c r="B20" t="str">
         <v>{{UPSELL_FEATURE_2}}</v>
       </c>
+      <c r="C20" t="str">
+        <v>contains</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -5323,6 +5341,9 @@
       <c r="B21" t="str">
         <v>{{UPSELL_FEATURE_3}}</v>
       </c>
+      <c r="C21" t="str">
+        <v>contains</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -5339,10 +5360,13 @@
       <c r="B23" t="str">
         <v>{{PPV_CTA_TEXT}}</v>
       </c>
+      <c r="C23" t="str">
+        <v>contains</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C23"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: enable max-parallel 4 and restore Home page sheet in PPV_Input
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Upgrade Confirmation page" sheetId="10" r:id="rId10"/>
     <sheet name="Phone Number page" sheetId="11" r:id="rId11"/>
     <sheet name="OTP page" sheetId="12" r:id="rId12"/>
+    <sheet name="Home page" sheetId="13" r:id="rId13"/>
   </sheets>
 </workbook>
 </file>
@@ -854,6 +855,84 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C6"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Flow</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Field</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Expected</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B2" t="str">
+        <v>The Biggest Fights Heading</v>
+      </c>
+      <c r="C2" t="str">
+        <v>The Biggest Fights</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B3" t="str">
+        <v>PPV Name</v>
+      </c>
+      <c r="C3" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B4" t="str">
+        <v>PPV Date and Time Text</v>
+      </c>
+      <c r="C4" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B5" t="str">
+        <v>PPV Image Present</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Buy Now CTA</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Buy now</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C55"/>

</xml_diff>

<commit_message>
feat: add mobile automation handoff flows, Android browser fixes, recording, validation helper stubs, and test support configurations
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -415,11 +415,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C12"/>
   <cols>
     <col min="1" max="1" width="33.83203125" customWidth="1"/>
     <col min="2" max="2" width="27.83203125" customWidth="1"/>
-    <col min="3" max="3" width="9.83203125" customWidth="1"/>
+    <col min="3" max="3" width="21.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -460,7 +460,7 @@
         <v>PPV Name</v>
       </c>
       <c r="B4" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{PPV_FULL_NAME}}</v>
       </c>
       <c r="C4" t="str">
         <v>landing</v>
@@ -488,9 +488,75 @@
         <v>landing</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Banner - Event Title</v>
+      </c>
+      <c r="B7" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+      <c r="C7" t="str">
+        <v>landing-page-banner</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Banner - Event Date</v>
+      </c>
+      <c r="B8" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+      <c r="C8" t="str">
+        <v>landing-page-banner</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Banner - Event Description</v>
+      </c>
+      <c r="B9" t="str">
+        <v>{{PPV_DESCRIPTION}}</v>
+      </c>
+      <c r="C9" t="str">
+        <v>landing-page-banner</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Banner Image Present</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C10" t="str">
+        <v>landing-page-banner</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Banner - Buy Now CTA</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Visible</v>
+      </c>
+      <c r="C11" t="str">
+        <v>landing-page-banner</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Banner - Fight Card CTA</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Visible</v>
+      </c>
+      <c r="C12" t="str">
+        <v>landing-page-banner</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -501,7 +567,7 @@
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
-    <col min="3" max="3" width="50.83203125" customWidth="1"/>
+    <col min="3" max="3" width="233.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -534,7 +600,7 @@
         <v>Page Description</v>
       </c>
       <c r="C3" t="str">
-        <v>Yes</v>
+        <v>All the action in one subscription. 12 pay-per-view fights a year with the ultimate viewing experience, plus football, basketball and more.</v>
       </c>
     </row>
     <row r="4">
@@ -572,24 +638,24 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>common</v>
+        <v>annual pay upfront</v>
       </c>
       <c r="B7" t="str">
         <v>Legal Text Line 1</v>
       </c>
       <c r="C7" t="str">
-        <v>Your plan will be changed to DAZN Ultimate today</v>
+        <v>Your plan will be changed to DAZN Ultimate today {{TODAY_DATE}} and your contract will last 12 months.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>common</v>
+        <v>annual pay upfront</v>
       </c>
       <c r="B8" t="str">
         <v>Legal Text Line 2</v>
       </c>
       <c r="C8" t="str">
-        <v>Today you will be charged</v>
+        <v>Today you will be charged {{CURRENCY}}{{ANNUAL_UPFRONT_PRICE}} minus the remainder of your last payment which was not used in full. From {{NEXT_PAYMENT_DATE}} you will be charged {{CURRENCY}}{{ANNUAL_UPFRONT_PRICE}}/year.</v>
       </c>
     </row>
     <row r="9">
@@ -644,7 +710,7 @@
         <v>Next Payment Label</v>
       </c>
       <c r="C13" t="str">
-        <v>Next payment on</v>
+        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
     </row>
     <row r="14">
@@ -660,13 +726,13 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>annual pay upfront</v>
+        <v>annual pay monthly</v>
       </c>
       <c r="B15" t="str">
-        <v>Next Payment Price</v>
+        <v>Legal Text Line 1</v>
       </c>
       <c r="C15" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
+        <v>Your plan will be changed to DAZN Ultimate today {{TODAY_DATE}} and your contract will last 12 months.</v>
       </c>
     </row>
     <row r="16">
@@ -674,10 +740,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B16" t="str">
-        <v>Rate Plan</v>
+        <v>Legal Text Line 2</v>
       </c>
       <c r="C16" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>Today you will be charged {{CURRENCY}}{{ANNUAL_PAY_MONTHLY_PRICE}} minus the remainder of your last payment which was not used in full. From {{NEXT_PAYMENT_DATE}} you will be charged {{CURRENCY}}{{ANNUAL_PAY_MONTHLY_PRICE}} /month.</v>
       </c>
     </row>
     <row r="17">
@@ -685,10 +751,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B17" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="C17" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
+        <v>Annual - Pay Monthly</v>
       </c>
     </row>
     <row r="18">
@@ -696,10 +762,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B18" t="str">
-        <v>Rate Plan Period</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="C18" t="str">
-        <v>/ month</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
     </row>
     <row r="19">
@@ -707,10 +773,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B19" t="str">
-        <v>Rate Plan Description</v>
+        <v>Rate Plan Period</v>
       </c>
       <c r="C19" t="str">
-        <v>Annual contract. Paid in 12 monthly instalments.</v>
+        <v>/ month</v>
       </c>
     </row>
     <row r="20">
@@ -718,10 +784,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B20" t="str">
-        <v>Next Payment Label</v>
+        <v>Rate Plan Description</v>
       </c>
       <c r="C20" t="str">
-        <v>Next payment on</v>
+        <v>Annual contract. Paid in 12 monthly instalments.</v>
       </c>
     </row>
     <row r="21">
@@ -729,10 +795,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B21" t="str">
-        <v>Next Payment Date</v>
+        <v>Next Payment Label</v>
       </c>
       <c r="C21" t="str">
-        <v>{{NEXT_PAYMENT_DATE}}</v>
+        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
     </row>
     <row r="22">
@@ -740,10 +806,10 @@
         <v>annual pay monthly</v>
       </c>
       <c r="B22" t="str">
-        <v>Next Payment Price</v>
+        <v>Next Payment Date</v>
       </c>
       <c r="C22" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
+        <v>{{NEXT_PAYMENT_DATE}}</v>
       </c>
     </row>
   </sheetData>
@@ -1051,11 +1117,11 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C19"/>
   <cols>
     <col min="1" max="1" width="21.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
-    <col min="3" max="3" width="21.83203125" customWidth="1"/>
+    <col min="3" max="3" width="90.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1176,7 +1242,7 @@
         <v>Popup - Event Description</v>
       </c>
       <c r="C11" t="str">
-        <v>{{PPV_DESCRIPTION}}</v>
+        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
       </c>
     </row>
     <row r="12">
@@ -1190,9 +1256,86 @@
         <v>Visible</v>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Biggest Fights Section</v>
+      </c>
+      <c r="C13" t="str">
+        <v>The Biggest Fights|Saturday Fight Night|Fight Night|Upcoming Big Fights|Big Fights</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Popup - Event Title</v>
+      </c>
+      <c r="C14" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Popup - Event Date</v>
+      </c>
+      <c r="C15" t="str">
+        <v>{{PPV_DATE}}</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Popup - Promoter</v>
+      </c>
+      <c r="C16" t="str">
+        <v>{{PPV_PROMOTER}}</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Popup - Buy Now CTA</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Popup - Event Description</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>home-biggest-fights</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Popup - Close Button</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Visible</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C19"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2477,7 +2620,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D102"/>
+  <dimension ref="A1:D94"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="37.83203125" customWidth="1"/>
@@ -2532,10 +2675,10 @@
         <v>variant1</v>
       </c>
       <c r="B4" t="str">
-        <v>Header Highlight Text1</v>
+        <v>Header Highlight Text2</v>
       </c>
       <c r="C4" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>N/A</v>
       </c>
       <c r="D4" t="str">
         <v/>
@@ -2546,10 +2689,10 @@
         <v>variant1</v>
       </c>
       <c r="B5" t="str">
-        <v>Header Highlight Text2</v>
+        <v>Event Name</v>
       </c>
       <c r="C5" t="str">
-        <v>N/A</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="D5" t="str">
         <v/>
@@ -2560,10 +2703,10 @@
         <v>variant1</v>
       </c>
       <c r="B6" t="str">
-        <v>Hero Image</v>
+        <v>PPV Per Fight Text</v>
       </c>
       <c r="C6" t="str">
-        <v>Yes</v>
+        <v>/fight</v>
       </c>
       <c r="D6" t="str">
         <v/>
@@ -2574,10 +2717,10 @@
         <v>variant1</v>
       </c>
       <c r="B7" t="str">
-        <v>Event Name</v>
+        <v>PPV Price</v>
       </c>
       <c r="C7" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{PPV_PRICE}}</v>
       </c>
       <c r="D7" t="str">
         <v/>
@@ -2588,10 +2731,10 @@
         <v>variant1</v>
       </c>
       <c r="B8" t="str">
-        <v>PPV Price</v>
+        <v>Currency</v>
       </c>
       <c r="C8" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>{{CURRENCY}}</v>
       </c>
       <c r="D8" t="str">
         <v/>
@@ -2602,13 +2745,13 @@
         <v>variant1</v>
       </c>
       <c r="B9" t="str">
-        <v>Currency</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="C9" t="str">
-        <v>{{CURRENCY}}</v>
+        <v>+DAZN Standard</v>
       </c>
       <c r="D9" t="str">
-        <v/>
+        <v>newuser</v>
       </c>
     </row>
     <row r="10">
@@ -2616,13 +2759,13 @@
         <v>variant1</v>
       </c>
       <c r="B10" t="str">
-        <v>DAZN Tier</v>
+        <v>PPV Name</v>
       </c>
       <c r="C10" t="str">
-        <v>+DAZN Standard</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="D10" t="str">
-        <v>newuser</v>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -2630,10 +2773,10 @@
         <v>variant1</v>
       </c>
       <c r="B11" t="str">
-        <v>PPV Name</v>
+        <v>PPV Image Present</v>
       </c>
       <c r="C11" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>Yes</v>
       </c>
       <c r="D11" t="str">
         <v/>
@@ -2644,10 +2787,10 @@
         <v>variant1</v>
       </c>
       <c r="B12" t="str">
-        <v>PPV Image Present</v>
+        <v>PPV Date and Time Text</v>
       </c>
       <c r="C12" t="str">
-        <v>Yes</v>
+        <v>{{PPV_DATE}}</v>
       </c>
       <c r="D12" t="str">
         <v/>
@@ -2658,10 +2801,10 @@
         <v>variant1</v>
       </c>
       <c r="B13" t="str">
-        <v>PPV Date and Time Text</v>
+        <v>Radio Selected</v>
       </c>
       <c r="C13" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>Yes</v>
       </c>
       <c r="D13" t="str">
         <v/>
@@ -2672,10 +2815,10 @@
         <v>variant1</v>
       </c>
       <c r="B14" t="str">
-        <v>Radio Selected</v>
+        <v>PPV Card Title</v>
       </c>
       <c r="C14" t="str">
-        <v>Yes</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="D14" t="str">
         <v/>
@@ -2686,10 +2829,10 @@
         <v>variant1</v>
       </c>
       <c r="B15" t="str">
-        <v>PPV Card Title</v>
+        <v>PPV Card Description</v>
       </c>
       <c r="C15" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{PPV_CARD_DESCRIPTION}}</v>
       </c>
       <c r="D15" t="str">
         <v/>
@@ -2700,10 +2843,10 @@
         <v>variant1</v>
       </c>
       <c r="B16" t="str">
-        <v>PPV Card Description</v>
+        <v>Upsell Section Present</v>
       </c>
       <c r="C16" t="str">
-        <v>{{PPV_CARD_DESCRIPTION}}</v>
+        <v>Yes</v>
       </c>
       <c r="D16" t="str">
         <v/>
@@ -2714,10 +2857,10 @@
         <v>variant1</v>
       </c>
       <c r="B17" t="str">
-        <v>Upsell Section Present</v>
+        <v>Upsell Badge</v>
       </c>
       <c r="C17" t="str">
-        <v>Yes</v>
+        <v>The Ultimate Fan Package</v>
       </c>
       <c r="D17" t="str">
         <v/>
@@ -2728,10 +2871,10 @@
         <v>variant1</v>
       </c>
       <c r="B18" t="str">
-        <v>Upsell Badge</v>
+        <v>Upsell Plan Name</v>
       </c>
       <c r="C18" t="str">
-        <v>The Ultimate Fan Package</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="D18" t="str">
         <v/>
@@ -2742,10 +2885,10 @@
         <v>variant1</v>
       </c>
       <c r="B19" t="str">
-        <v>Upsell Plan Name</v>
+        <v>Upsell Price Text</v>
       </c>
       <c r="C19" t="str">
-        <v>DAZN Ultimate</v>
+        <v>N/A</v>
       </c>
       <c r="D19" t="str">
         <v/>
@@ -2756,10 +2899,10 @@
         <v>variant1</v>
       </c>
       <c r="B20" t="str">
-        <v>Upsell Price Text</v>
+        <v>Upsell Price</v>
       </c>
       <c r="C20" t="str">
-        <v>N/A</v>
+        <v>{{UPSELL_PRICE}}</v>
       </c>
       <c r="D20" t="str">
         <v/>
@@ -2770,10 +2913,10 @@
         <v>variant1</v>
       </c>
       <c r="B21" t="str">
-        <v>Upsell Price</v>
+        <v>Upsell Price Length</v>
       </c>
       <c r="C21" t="str">
-        <v>{{UPSELL_PRICE}}</v>
+        <v>{{UPSELL_PRICE_LENGTH}}</v>
       </c>
       <c r="D21" t="str">
         <v/>
@@ -2784,10 +2927,10 @@
         <v>variant1</v>
       </c>
       <c r="B22" t="str">
-        <v>Upsell Price Length</v>
+        <v>Upsell Crossed Price</v>
       </c>
       <c r="C22" t="str">
-        <v>{{UPSELL_PRICE_LENGTH}}</v>
+        <v>{{UPSELL_CROSSED_PRICE}}</v>
       </c>
       <c r="D22" t="str">
         <v/>
@@ -2798,10 +2941,10 @@
         <v>variant1</v>
       </c>
       <c r="B23" t="str">
-        <v>Upsell Crossed Price</v>
+        <v>Upsell Billing Text</v>
       </c>
       <c r="C23" t="str">
-        <v>{{UPSELL_CROSSED_PRICE}}</v>
+        <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
       </c>
       <c r="D23" t="str">
         <v/>
@@ -2812,13 +2955,13 @@
         <v>variant1</v>
       </c>
       <c r="B24" t="str">
-        <v>Upsell Contract Text</v>
+        <v>Upsell Offer Text</v>
       </c>
       <c r="C24" t="str">
-        <v>Annual contract. Auto renews.</v>
+        <v>{{UPSELL_OFFER_TEXT}}</v>
       </c>
       <c r="D24" t="str">
-        <v/>
+        <v>offer</v>
       </c>
     </row>
     <row r="25">
@@ -2826,10 +2969,10 @@
         <v>variant1</v>
       </c>
       <c r="B25" t="str">
-        <v>Upsell Billing Text</v>
+        <v>Upsell Section Heading</v>
       </c>
       <c r="C25" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_CONTRACT_TEXT}}</v>
+        <v>{{UPSELL_SECTION_HEADING}}</v>
       </c>
       <c r="D25" t="str">
         <v/>
@@ -2840,13 +2983,13 @@
         <v>variant1</v>
       </c>
       <c r="B26" t="str">
-        <v>Upsell Offer Text</v>
+        <v>PPV1 Included tag</v>
       </c>
       <c r="C26" t="str">
-        <v>{{UPSELL_OFFER_TEXT}}</v>
+        <v>N/A</v>
       </c>
       <c r="D26" t="str">
-        <v>offer</v>
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -2854,10 +2997,10 @@
         <v>variant1</v>
       </c>
       <c r="B27" t="str">
-        <v>Upsell Section Heading</v>
+        <v>Included PPV2 Name</v>
       </c>
       <c r="C27" t="str">
-        <v>{{UPSELL_SECTION_HEADING}}</v>
+        <v>N/A</v>
       </c>
       <c r="D27" t="str">
         <v/>
@@ -2868,10 +3011,10 @@
         <v>variant1</v>
       </c>
       <c r="B28" t="str">
-        <v>Included PPV1 Name</v>
+        <v>PPV2 Image Present on ultimate tier</v>
       </c>
       <c r="C28" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>N/A</v>
       </c>
       <c r="D28" t="str">
         <v/>
@@ -2882,10 +3025,10 @@
         <v>variant1</v>
       </c>
       <c r="B29" t="str">
-        <v>PPV1 Image Present on ultimate tier</v>
+        <v>PPV2 Date Text on ultimate tier</v>
       </c>
       <c r="C29" t="str">
-        <v>Yes</v>
+        <v>N/A</v>
       </c>
       <c r="D29" t="str">
         <v/>
@@ -2896,10 +3039,10 @@
         <v>variant1</v>
       </c>
       <c r="B30" t="str">
-        <v>PPV1 Upsell Tile Date</v>
+        <v>PPV2 Included tag</v>
       </c>
       <c r="C30" t="str">
-        <v>{{PPV1_UPSELL_TILE_DATE}}</v>
+        <v>N/A</v>
       </c>
       <c r="D30" t="str">
         <v/>
@@ -2910,10 +3053,10 @@
         <v>variant1</v>
       </c>
       <c r="B31" t="str">
-        <v>PPV1 Included tag</v>
+        <v>Upsell Feature 1</v>
       </c>
       <c r="C31" t="str">
-        <v>N/A</v>
+        <v>{{UPSELL_FEATURE_1}}</v>
       </c>
       <c r="D31" t="str">
         <v/>
@@ -2924,7 +3067,7 @@
         <v>variant1</v>
       </c>
       <c r="B32" t="str">
-        <v>Included PPV2 Name</v>
+        <v>Upsell Highlight Text</v>
       </c>
       <c r="C32" t="str">
         <v>N/A</v>
@@ -2938,10 +3081,10 @@
         <v>variant1</v>
       </c>
       <c r="B33" t="str">
-        <v>PPV2 Image Present on ultimate tier</v>
+        <v>Upsell Feature 2</v>
       </c>
       <c r="C33" t="str">
-        <v>N/A</v>
+        <v>{{UPSELL_FEATURE_2}}</v>
       </c>
       <c r="D33" t="str">
         <v/>
@@ -2952,10 +3095,10 @@
         <v>variant1</v>
       </c>
       <c r="B34" t="str">
-        <v>PPV2 Date Text on ultimate tier</v>
+        <v>Upsell Feature 3</v>
       </c>
       <c r="C34" t="str">
-        <v>N/A</v>
+        <v>{{UPSELL_FEATURE_3}}</v>
       </c>
       <c r="D34" t="str">
         <v/>
@@ -2966,7 +3109,7 @@
         <v>variant1</v>
       </c>
       <c r="B35" t="str">
-        <v>PPV2 Included tag</v>
+        <v>Whats Included CTA</v>
       </c>
       <c r="C35" t="str">
         <v>N/A</v>
@@ -2980,10 +3123,10 @@
         <v>variant1</v>
       </c>
       <c r="B36" t="str">
-        <v>Upsell Feature 1</v>
+        <v>Gold Highlight 1</v>
       </c>
       <c r="C36" t="str">
-        <v>{{UPSELL_FEATURE_1}}</v>
+        <v>N/A</v>
       </c>
       <c r="D36" t="str">
         <v/>
@@ -2994,7 +3137,7 @@
         <v>variant1</v>
       </c>
       <c r="B37" t="str">
-        <v>Upsell Highlight Text</v>
+        <v>Gold Highlight 2</v>
       </c>
       <c r="C37" t="str">
         <v>N/A</v>
@@ -3008,10 +3151,10 @@
         <v>variant1</v>
       </c>
       <c r="B38" t="str">
-        <v>Upsell Feature 2</v>
+        <v>Gold Highlight 3</v>
       </c>
       <c r="C38" t="str">
-        <v>{{UPSELL_FEATURE_2}}</v>
+        <v>N/A</v>
       </c>
       <c r="D38" t="str">
         <v/>
@@ -3022,13 +3165,13 @@
         <v>variant1</v>
       </c>
       <c r="B39" t="str">
-        <v>Upsell Feature 3</v>
+        <v>Bundle Name</v>
       </c>
       <c r="C39" t="str">
-        <v>{{UPSELL_FEATURE_3}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="D39" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="40">
@@ -3036,13 +3179,13 @@
         <v>variant1</v>
       </c>
       <c r="B40" t="str">
-        <v>Whats Included CTA</v>
+        <v>Bundle Description</v>
       </c>
       <c r="C40" t="str">
-        <v>N/A</v>
+        <v>{{BUNDLE_DESCRIPTION}}</v>
       </c>
       <c r="D40" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="41">
@@ -3050,13 +3193,13 @@
         <v>variant1</v>
       </c>
       <c r="B41" t="str">
-        <v>Gold Highlight 1</v>
+        <v>Bundle Monthly Price</v>
       </c>
       <c r="C41" t="str">
-        <v>N/A</v>
+        <v>{{BUNDLE_MONTHLY_PRICE}}</v>
       </c>
       <c r="D41" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="42">
@@ -3064,13 +3207,13 @@
         <v>variant1</v>
       </c>
       <c r="B42" t="str">
-        <v>Gold Highlight 2</v>
+        <v>Bundle Price</v>
       </c>
       <c r="C42" t="str">
-        <v>N/A</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="D42" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="43">
@@ -3078,13 +3221,13 @@
         <v>variant1</v>
       </c>
       <c r="B43" t="str">
-        <v>Gold Highlight 3</v>
+        <v>Bundle Original Price</v>
       </c>
       <c r="C43" t="str">
-        <v>N/A</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="D43" t="str">
-        <v/>
+        <v>bundle</v>
       </c>
     </row>
     <row r="44">
@@ -3092,10 +3235,10 @@
         <v>variant1</v>
       </c>
       <c r="B44" t="str">
-        <v>Bundle Name</v>
+        <v>Bundle Fight Count</v>
       </c>
       <c r="C44" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>{{BUNDLE_FIGHT_COUNT}}</v>
       </c>
       <c r="D44" t="str">
         <v>bundle</v>
@@ -3106,10 +3249,10 @@
         <v>variant1</v>
       </c>
       <c r="B45" t="str">
-        <v>Bundle Description</v>
+        <v>Bundle Save Badge</v>
       </c>
       <c r="C45" t="str">
-        <v>{{BUNDLE_DESCRIPTION}}</v>
+        <v>{{BUNDLE_SAVE_BADGE}}</v>
       </c>
       <c r="D45" t="str">
         <v>bundle</v>
@@ -3120,10 +3263,10 @@
         <v>variant1</v>
       </c>
       <c r="B46" t="str">
-        <v>Bundle Monthly Price</v>
+        <v>Bundle PPV 1 Full Name</v>
       </c>
       <c r="C46" t="str">
-        <v>{{BUNDLE_MONTHLY_PRICE}}</v>
+        <v>{{BUNDLE_PPV1_FULL_NAME}}</v>
       </c>
       <c r="D46" t="str">
         <v>bundle</v>
@@ -3134,10 +3277,10 @@
         <v>variant1</v>
       </c>
       <c r="B47" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle PPV 1 Date</v>
       </c>
       <c r="C47" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>{{BUNDLE_PPV1_DATE}}</v>
       </c>
       <c r="D47" t="str">
         <v>bundle</v>
@@ -3148,10 +3291,10 @@
         <v>variant1</v>
       </c>
       <c r="B48" t="str">
-        <v>Bundle Original Price</v>
+        <v>Bundle PPV 1 Image</v>
       </c>
       <c r="C48" t="str">
-        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
+        <v>Yes</v>
       </c>
       <c r="D48" t="str">
         <v>bundle</v>
@@ -3162,10 +3305,10 @@
         <v>variant1</v>
       </c>
       <c r="B49" t="str">
-        <v>Bundle Fight Count</v>
+        <v>Bundle PPV 2 Full Name</v>
       </c>
       <c r="C49" t="str">
-        <v>{{BUNDLE_FIGHT_COUNT}}</v>
+        <v>{{BUNDLE_PPV2_FULL_NAME}}</v>
       </c>
       <c r="D49" t="str">
         <v>bundle</v>
@@ -3176,10 +3319,10 @@
         <v>variant1</v>
       </c>
       <c r="B50" t="str">
-        <v>Bundle Save Badge</v>
+        <v>Bundle PPV 2 Date</v>
       </c>
       <c r="C50" t="str">
-        <v>{{BUNDLE_SAVE_BADGE}}</v>
+        <v>{{BUNDLE_PPV2_DATE}}</v>
       </c>
       <c r="D50" t="str">
         <v>bundle</v>
@@ -3190,10 +3333,10 @@
         <v>variant1</v>
       </c>
       <c r="B51" t="str">
-        <v>Bundle PPV 1 Full Name</v>
+        <v>Bundle PPV 2 Image</v>
       </c>
       <c r="C51" t="str">
-        <v>{{BUNDLE_PPV1_FULL_NAME}}</v>
+        <v>Yes</v>
       </c>
       <c r="D51" t="str">
         <v>bundle</v>
@@ -3204,13 +3347,13 @@
         <v>variant1</v>
       </c>
       <c r="B52" t="str">
-        <v>Bundle PPV 1 Date</v>
+        <v>CTA Button</v>
       </c>
       <c r="C52" t="str">
-        <v>{{BUNDLE_PPV1_DATE}}</v>
+        <v>{{PPV_CTA_TEXT}}</v>
       </c>
       <c r="D52" t="str">
-        <v>bundle</v>
+        <v/>
       </c>
     </row>
     <row r="53">
@@ -3218,66 +3361,66 @@
         <v>variant1</v>
       </c>
       <c r="B53" t="str">
-        <v>Bundle PPV 1 Image</v>
+        <v>CTA Without PPV</v>
       </c>
       <c r="C53" t="str">
-        <v>Yes</v>
+        <v>Subscribe without a pay-per-view</v>
       </c>
       <c r="D53" t="str">
-        <v>bundle</v>
+        <v>newuser</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>variant1</v>
+        <v>variant2</v>
       </c>
       <c r="B54" t="str">
-        <v>Bundle PPV 2 Full Name</v>
+        <v>Page Title</v>
       </c>
       <c r="C54" t="str">
-        <v>{{BUNDLE_PPV2_FULL_NAME}}</v>
+        <v>Choose your plan</v>
       </c>
       <c r="D54" t="str">
-        <v>bundle</v>
+        <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>variant1</v>
+        <v>variant2</v>
       </c>
       <c r="B55" t="str">
-        <v>Bundle PPV 2 Date</v>
+        <v>Header Full Copy</v>
       </c>
       <c r="C55" t="str">
-        <v>{{BUNDLE_PPV2_DATE}}</v>
+        <v>Buy {{PPV_NAME}} with DAZN Standard or get it included in DAZN Ultimate.</v>
       </c>
       <c r="D55" t="str">
-        <v>bundle</v>
+        <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>variant1</v>
+        <v>variant2</v>
       </c>
       <c r="B56" t="str">
-        <v>Bundle PPV 2 Image</v>
+        <v>Header Highlight Text2</v>
       </c>
       <c r="C56" t="str">
-        <v>Yes</v>
+        <v>get it included in DAZN Ultimate.</v>
       </c>
       <c r="D56" t="str">
-        <v>bundle</v>
+        <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>variant1</v>
+        <v>variant2</v>
       </c>
       <c r="B57" t="str">
-        <v>CTA Button</v>
+        <v>PPV Image</v>
       </c>
       <c r="C57" t="str">
-        <v>{{PPV_CTA_TEXT}}</v>
+        <v>Yes</v>
       </c>
       <c r="D57" t="str">
         <v/>
@@ -3285,16 +3428,16 @@
     </row>
     <row r="58">
       <c r="A58" t="str">
-        <v>variant1</v>
+        <v>variant2</v>
       </c>
       <c r="B58" t="str">
-        <v>CTA Without PPV</v>
+        <v>Event Date and Time</v>
       </c>
       <c r="C58" t="str">
-        <v>Subscribe without a pay-per-view</v>
+        <v>{{PPV_DATE}}</v>
       </c>
       <c r="D58" t="str">
-        <v>newuser</v>
+        <v/>
       </c>
     </row>
     <row r="59">
@@ -3302,10 +3445,10 @@
         <v>variant2</v>
       </c>
       <c r="B59" t="str">
-        <v>Page Title</v>
+        <v>Event Name</v>
       </c>
       <c r="C59" t="str">
-        <v>Choose your plan</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="D59" t="str">
         <v/>
@@ -3316,10 +3459,10 @@
         <v>variant2</v>
       </c>
       <c r="B60" t="str">
-        <v>Header Full Copy</v>
+        <v>PPV Checkbox Present</v>
       </c>
       <c r="C60" t="str">
-        <v>Buy {{PPV_NAME}} with DAZN Standard or get it included in DAZN Ultimate.</v>
+        <v>Yes</v>
       </c>
       <c r="D60" t="str">
         <v/>
@@ -3330,10 +3473,10 @@
         <v>variant2</v>
       </c>
       <c r="B61" t="str">
-        <v>Header Highlight Text1</v>
+        <v>PPV Selected</v>
       </c>
       <c r="C61" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>Yes</v>
       </c>
       <c r="D61" t="str">
         <v/>
@@ -3344,10 +3487,10 @@
         <v>variant2</v>
       </c>
       <c r="B62" t="str">
-        <v>Header Highlight Text2</v>
+        <v>PPV Name</v>
       </c>
       <c r="C62" t="str">
-        <v>get it included in DAZN Ultimate.</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="D62" t="str">
         <v/>
@@ -3358,10 +3501,10 @@
         <v>variant2</v>
       </c>
       <c r="B63" t="str">
-        <v>PPV Image</v>
+        <v>PPV Per Fight Text</v>
       </c>
       <c r="C63" t="str">
-        <v>Yes</v>
+        <v>/fight</v>
       </c>
       <c r="D63" t="str">
         <v/>
@@ -3372,10 +3515,10 @@
         <v>variant2</v>
       </c>
       <c r="B64" t="str">
-        <v>Event Date and Time</v>
+        <v>PPV Price</v>
       </c>
       <c r="C64" t="str">
-        <v>{{PPV_DATE}}</v>
+        <v>{{PPV_PRICE}}</v>
       </c>
       <c r="D64" t="str">
         <v/>
@@ -3386,10 +3529,10 @@
         <v>variant2</v>
       </c>
       <c r="B65" t="str">
-        <v>Event Name</v>
+        <v>Currency</v>
       </c>
       <c r="C65" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{CURRENCY}}</v>
       </c>
       <c r="D65" t="str">
         <v/>
@@ -3400,10 +3543,10 @@
         <v>variant2</v>
       </c>
       <c r="B66" t="str">
-        <v>PPV Checkbox Present</v>
+        <v>Subscription Section Title</v>
       </c>
       <c r="C66" t="str">
-        <v>Yes</v>
+        <v>Choose your subscription</v>
       </c>
       <c r="D66" t="str">
         <v/>
@@ -3414,7 +3557,7 @@
         <v>variant2</v>
       </c>
       <c r="B67" t="str">
-        <v>PPV Selected</v>
+        <v>Trial Card Present</v>
       </c>
       <c r="C67" t="str">
         <v>Yes</v>
@@ -3428,10 +3571,10 @@
         <v>variant2</v>
       </c>
       <c r="B68" t="str">
-        <v>PPV Name</v>
+        <v>Trial Title</v>
       </c>
       <c r="C68" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>7-day free trial of DAZN Standard</v>
       </c>
       <c r="D68" t="str">
         <v/>
@@ -3442,10 +3585,10 @@
         <v>variant2</v>
       </c>
       <c r="B69" t="str">
-        <v>PPV Price</v>
+        <v>Trial Radio Present</v>
       </c>
       <c r="C69" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>Yes</v>
       </c>
       <c r="D69" t="str">
         <v/>
@@ -3456,10 +3599,10 @@
         <v>variant2</v>
       </c>
       <c r="B70" t="str">
-        <v>Currency</v>
+        <v>Trial Selected</v>
       </c>
       <c r="C70" t="str">
-        <v>{{CURRENCY}}</v>
+        <v>Yes</v>
       </c>
       <c r="D70" t="str">
         <v/>
@@ -3470,10 +3613,10 @@
         <v>variant2</v>
       </c>
       <c r="B71" t="str">
-        <v>Subscription Section Title</v>
+        <v>Trial Feature 1</v>
       </c>
       <c r="C71" t="str">
-        <v>Choose your subscription</v>
+        <v>7-days free access to DAZN Standard.</v>
       </c>
       <c r="D71" t="str">
         <v/>
@@ -3484,10 +3627,10 @@
         <v>variant2</v>
       </c>
       <c r="B72" t="str">
-        <v>Trial Card Present</v>
+        <v>Trial Feature 2</v>
       </c>
       <c r="C72" t="str">
-        <v>Yes</v>
+        <v>Cancel anytime during the trial and only pay for the fight. After the trial you move onto a Monthly Flex plan for {{CURRENCY}}{{MONTHLY_PRICE}}/month. You will not lose access to the pay-per-view[s].</v>
       </c>
       <c r="D72" t="str">
         <v/>
@@ -3498,10 +3641,10 @@
         <v>variant2</v>
       </c>
       <c r="B73" t="str">
-        <v>Trial Title</v>
+        <v>Upsell Section Present</v>
       </c>
       <c r="C73" t="str">
-        <v>7-day free trial of DAZN Standard</v>
+        <v>Yes</v>
       </c>
       <c r="D73" t="str">
         <v/>
@@ -3512,10 +3655,10 @@
         <v>variant2</v>
       </c>
       <c r="B74" t="str">
-        <v>Trial Radio Present</v>
+        <v>Upsell Label</v>
       </c>
       <c r="C74" t="str">
-        <v>Yes</v>
+        <v>Pay-per-views included</v>
       </c>
       <c r="D74" t="str">
         <v/>
@@ -3526,10 +3669,10 @@
         <v>variant2</v>
       </c>
       <c r="B75" t="str">
-        <v>Trial Selected</v>
+        <v>Upsell Plan Name</v>
       </c>
       <c r="C75" t="str">
-        <v>Yes</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="D75" t="str">
         <v/>
@@ -3540,10 +3683,10 @@
         <v>variant2</v>
       </c>
       <c r="B76" t="str">
-        <v>Trial Feature 1</v>
+        <v>Upsell Price Text</v>
       </c>
       <c r="C76" t="str">
-        <v>7-days free access to DAZN Standard.</v>
+        <v>From</v>
       </c>
       <c r="D76" t="str">
         <v/>
@@ -3554,10 +3697,10 @@
         <v>variant2</v>
       </c>
       <c r="B77" t="str">
-        <v>Trial Feature 2</v>
+        <v>Upsell Price</v>
       </c>
       <c r="C77" t="str">
-        <v>Cancel anytime during the trial and only pay for the fight. After the trial you move onto a Monthly Flex plan for {{CURRENCY}}{{MONTHLY_PRICE}}/month. You will not lose access to the pay-per-view[s].</v>
+        <v>{{UPSELL_PRICE}}</v>
       </c>
       <c r="D77" t="str">
         <v/>
@@ -3568,10 +3711,10 @@
         <v>variant2</v>
       </c>
       <c r="B78" t="str">
-        <v>Upsell Section Present</v>
+        <v>Upsell Price Length</v>
       </c>
       <c r="C78" t="str">
-        <v>Yes</v>
+        <v>{{UPSELL_PRICE_LENGTH}}</v>
       </c>
       <c r="D78" t="str">
         <v/>
@@ -3582,10 +3725,10 @@
         <v>variant2</v>
       </c>
       <c r="B79" t="str">
-        <v>Upsell Label</v>
+        <v>Upsell Billing Text</v>
       </c>
       <c r="C79" t="str">
-        <v>Pay-per-views included</v>
+        <v>Annual contract. Auto renews.</v>
       </c>
       <c r="D79" t="str">
         <v/>
@@ -3596,10 +3739,10 @@
         <v>variant2</v>
       </c>
       <c r="B80" t="str">
-        <v>Upsell Plan Name</v>
+        <v>PPV1 Included tag</v>
       </c>
       <c r="C80" t="str">
-        <v>DAZN Ultimate</v>
+        <v>Yes</v>
       </c>
       <c r="D80" t="str">
         <v/>
@@ -3610,10 +3753,10 @@
         <v>variant2</v>
       </c>
       <c r="B81" t="str">
-        <v>Upsell Price Text</v>
+        <v>Included PPV2 Name</v>
       </c>
       <c r="C81" t="str">
-        <v>From</v>
+        <v>N/A</v>
       </c>
       <c r="D81" t="str">
         <v/>
@@ -3624,10 +3767,10 @@
         <v>variant2</v>
       </c>
       <c r="B82" t="str">
-        <v>Upsell Price</v>
+        <v>PPV2 Image Present on ultimate tier</v>
       </c>
       <c r="C82" t="str">
-        <v>{{UPSELL_PRICE}}</v>
+        <v>N/A</v>
       </c>
       <c r="D82" t="str">
         <v/>
@@ -3638,10 +3781,10 @@
         <v>variant2</v>
       </c>
       <c r="B83" t="str">
-        <v>Upsell Price Length</v>
+        <v>PPV2 Date Text on ultimate tier</v>
       </c>
       <c r="C83" t="str">
-        <v>{{UPSELL_PRICE_LENGTH}}</v>
+        <v>N/A</v>
       </c>
       <c r="D83" t="str">
         <v/>
@@ -3652,10 +3795,10 @@
         <v>variant2</v>
       </c>
       <c r="B84" t="str">
-        <v>Upsell Billing Text</v>
+        <v>PPV2 Included tag</v>
       </c>
       <c r="C84" t="str">
-        <v>Annual contract. Auto renews.</v>
+        <v>N/A</v>
       </c>
       <c r="D84" t="str">
         <v/>
@@ -3666,10 +3809,10 @@
         <v>variant2</v>
       </c>
       <c r="B85" t="str">
-        <v>Included PPV1 Name</v>
+        <v>Upsell Feature 1</v>
       </c>
       <c r="C85" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>Pay-per-views included at no extra cost. Minimum of 12 events per year including {{PPV_NAME}}.</v>
       </c>
       <c r="D85" t="str">
         <v/>
@@ -3680,10 +3823,10 @@
         <v>variant2</v>
       </c>
       <c r="B86" t="str">
-        <v>PPV1 Image Present on ultimate tier</v>
+        <v>Upsell Highlight Text</v>
       </c>
       <c r="C86" t="str">
-        <v>Yes</v>
+        <v>{{PPV_NAME}}.</v>
       </c>
       <c r="D86" t="str">
         <v/>
@@ -3694,10 +3837,10 @@
         <v>variant2</v>
       </c>
       <c r="B87" t="str">
-        <v>PPV1 Upsell Tile Date</v>
+        <v>Upsell Feature 2</v>
       </c>
       <c r="C87" t="str">
-        <v>{{PPV1_UPSELL_TILE_DATE}}</v>
+        <v>HDR and Dolby 5.1 surround sound on select events.</v>
       </c>
       <c r="D87" t="str">
         <v/>
@@ -3708,10 +3851,10 @@
         <v>variant2</v>
       </c>
       <c r="B88" t="str">
-        <v>PPV1 Included tag</v>
+        <v>Upsell Feature 3</v>
       </c>
       <c r="C88" t="str">
-        <v>Yes</v>
+        <v>185+ fights a year from the best promoters</v>
       </c>
       <c r="D88" t="str">
         <v/>
@@ -3722,10 +3865,10 @@
         <v>variant2</v>
       </c>
       <c r="B89" t="str">
-        <v>Included PPV2 Name</v>
+        <v>Whats Included CTA</v>
       </c>
       <c r="C89" t="str">
-        <v>N/A</v>
+        <v>Whats included</v>
       </c>
       <c r="D89" t="str">
         <v/>
@@ -3736,10 +3879,10 @@
         <v>variant2</v>
       </c>
       <c r="B90" t="str">
-        <v>PPV2 Image Present on ultimate tier</v>
+        <v>Gold Highlight 1</v>
       </c>
       <c r="C90" t="str">
-        <v>N/A</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="D90" t="str">
         <v/>
@@ -3750,10 +3893,10 @@
         <v>variant2</v>
       </c>
       <c r="B91" t="str">
-        <v>PPV2 Date Text on ultimate tier</v>
+        <v>Gold Highlight 2</v>
       </c>
       <c r="C91" t="str">
-        <v>N/A</v>
+        <v>get it included in DAZN Ultimate.</v>
       </c>
       <c r="D91" t="str">
         <v/>
@@ -3764,10 +3907,10 @@
         <v>variant2</v>
       </c>
       <c r="B92" t="str">
-        <v>PPV2 Included tag</v>
+        <v>Gold Highlight 3</v>
       </c>
       <c r="C92" t="str">
-        <v>N/A</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="D92" t="str">
         <v/>
@@ -3778,10 +3921,10 @@
         <v>variant2</v>
       </c>
       <c r="B93" t="str">
-        <v>Upsell Feature 1</v>
+        <v>CTA Button</v>
       </c>
       <c r="C93" t="str">
-        <v>Pay-per-views included at no extra cost. Minimum of 12 events per year including {{PPV_NAME}}.</v>
+        <v>Continue with PPV + 7-day free trial</v>
       </c>
       <c r="D93" t="str">
         <v/>
@@ -3792,130 +3935,18 @@
         <v>variant2</v>
       </c>
       <c r="B94" t="str">
-        <v>Upsell Highlight Text</v>
+        <v>CTA Without PPV</v>
       </c>
       <c r="C94" t="str">
-        <v>{{PPV_NAME}}.</v>
+        <v>N/A</v>
       </c>
       <c r="D94" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" t="str">
-        <v>variant2</v>
-      </c>
-      <c r="B95" t="str">
-        <v>Upsell Feature 2</v>
-      </c>
-      <c r="C95" t="str">
-        <v>HDR and Dolby 5.1 surround sound on select events.</v>
-      </c>
-      <c r="D95" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" t="str">
-        <v>variant2</v>
-      </c>
-      <c r="B96" t="str">
-        <v>Upsell Feature 3</v>
-      </c>
-      <c r="C96" t="str">
-        <v>185+ fights a year from the best promoters</v>
-      </c>
-      <c r="D96" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="str">
-        <v>variant2</v>
-      </c>
-      <c r="B97" t="str">
-        <v>Whats Included CTA</v>
-      </c>
-      <c r="C97" t="str">
-        <v>Whats included</v>
-      </c>
-      <c r="D97" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" t="str">
-        <v>variant2</v>
-      </c>
-      <c r="B98" t="str">
-        <v>Gold Highlight 1</v>
-      </c>
-      <c r="C98" t="str">
-        <v>{{PPV_NAME}}</v>
-      </c>
-      <c r="D98" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" t="str">
-        <v>variant2</v>
-      </c>
-      <c r="B99" t="str">
-        <v>Gold Highlight 2</v>
-      </c>
-      <c r="C99" t="str">
-        <v>get it included in DAZN Ultimate.</v>
-      </c>
-      <c r="D99" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" t="str">
-        <v>variant2</v>
-      </c>
-      <c r="B100" t="str">
-        <v>Gold Highlight 3</v>
-      </c>
-      <c r="C100" t="str">
-        <v>DAZN Ultimate</v>
-      </c>
-      <c r="D100" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" t="str">
-        <v>variant2</v>
-      </c>
-      <c r="B101" t="str">
-        <v>CTA Button</v>
-      </c>
-      <c r="C101" t="str">
-        <v>Continue with PPV + 7-day free trial</v>
-      </c>
-      <c r="D101" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" t="str">
-        <v>variant2</v>
-      </c>
-      <c r="B102" t="str">
-        <v>CTA Without PPV</v>
-      </c>
-      <c r="C102" t="str">
-        <v>N/A</v>
-      </c>
-      <c r="D102" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D102"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D94"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4457,7 +4488,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E102"/>
+  <dimension ref="A1:E103"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="27.83203125" customWidth="1"/>
@@ -4491,10 +4522,10 @@
         <v>All</v>
       </c>
       <c r="C2" t="str">
-        <v>Header</v>
+        <v>Payment Method Heading</v>
       </c>
       <c r="D2" t="str">
-        <v>Your payment is encrypted and you can change how you pay at any time.</v>
+        <v>Payment method</v>
       </c>
       <c r="E2" t="str">
         <v/>
@@ -4508,10 +4539,10 @@
         <v>All</v>
       </c>
       <c r="C3" t="str">
-        <v>Plan Change CTA</v>
+        <v>Purchase Summary Heading</v>
       </c>
       <c r="D3" t="str">
-        <v>Change</v>
+        <v>Purchase summary</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -4525,10 +4556,10 @@
         <v>All</v>
       </c>
       <c r="C4" t="str">
-        <v>Credit &amp; Debit Card Option</v>
+        <v>Plan Change CTA</v>
       </c>
       <c r="D4" t="str">
-        <v>Yes</v>
+        <v>Change</v>
       </c>
       <c r="E4" t="str">
         <v/>
@@ -4542,7 +4573,7 @@
         <v>All</v>
       </c>
       <c r="C5" t="str">
-        <v>PayPal Option</v>
+        <v>Credit &amp; Debit Card Option</v>
       </c>
       <c r="D5" t="str">
         <v>Yes</v>
@@ -4559,7 +4590,7 @@
         <v>All</v>
       </c>
       <c r="C6" t="str">
-        <v>Google Pay Option</v>
+        <v>PayPal Option</v>
       </c>
       <c r="D6" t="str">
         <v>Yes</v>
@@ -4576,13 +4607,13 @@
         <v>All</v>
       </c>
       <c r="C7" t="str">
-        <v>Saved Card Present</v>
+        <v>Google Pay Option</v>
       </c>
       <c r="D7" t="str">
         <v>Yes</v>
       </c>
       <c r="E7" t="str">
-        <v>myaccount</v>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -4593,13 +4624,13 @@
         <v>All</v>
       </c>
       <c r="C8" t="str">
-        <v>Signed In As Text</v>
+        <v>Saved Card Present</v>
       </c>
       <c r="D8" t="str">
-        <v>Signed in as {{FIRST_NAME}} {{LAST_NAME}}</v>
+        <v>Yes</v>
       </c>
       <c r="E8" t="str">
-        <v>returning</v>
+        <v>myaccount</v>
       </c>
     </row>
     <row r="9">
@@ -4610,10 +4641,10 @@
         <v>All</v>
       </c>
       <c r="C9" t="str">
-        <v>Log Out Present</v>
+        <v>Signed In As Text</v>
       </c>
       <c r="D9" t="str">
-        <v>Yes</v>
+        <v>Signed in as {{FIRST_NAME}} {{LAST_NAME}}</v>
       </c>
       <c r="E9" t="str">
         <v>returning</v>
@@ -4627,30 +4658,30 @@
         <v>All</v>
       </c>
       <c r="C10" t="str">
-        <v>Redeem Promo Code CTA</v>
+        <v>Log Out Present</v>
       </c>
       <c r="D10" t="str">
         <v>Yes</v>
       </c>
       <c r="E10" t="str">
-        <v/>
+        <v>returning</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Standard</v>
+        <v>Common</v>
       </c>
       <c r="B11" t="str">
-        <v>Monthly</v>
+        <v>All</v>
       </c>
       <c r="C11" t="str">
-        <v>Page Title</v>
+        <v>Redeem Promo Code CTA</v>
       </c>
       <c r="D11" t="str">
-        <v>{{PAYMENT_PAGE_TITLE}}</v>
+        <v>Yes</v>
       </c>
       <c r="E11" t="str">
-        <v>newuser</v>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -4667,7 +4698,7 @@
         <v>{{PAYMENT_PAGE_TITLE}}</v>
       </c>
       <c r="E12" t="str">
-        <v>myaccount</v>
+        <v>newuser</v>
       </c>
     </row>
     <row r="13">
@@ -4678,13 +4709,13 @@
         <v>Monthly</v>
       </c>
       <c r="C13" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D13" t="str">
-        <v>DAZN Standard</v>
+        <v>{{PAYMENT_PAGE_TITLE}}</v>
       </c>
       <c r="E13" t="str">
-        <v/>
+        <v>myaccount</v>
       </c>
     </row>
     <row r="14">
@@ -4695,10 +4726,10 @@
         <v>Monthly</v>
       </c>
       <c r="C14" t="str">
-        <v>Plan Name</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D14" t="str">
-        <v>{{PAYMENT_PLAN_NAME}}</v>
+        <v>DAZN Standard</v>
       </c>
       <c r="E14" t="str">
         <v/>
@@ -4712,10 +4743,10 @@
         <v>Monthly</v>
       </c>
       <c r="C15" t="str">
-        <v>Plan Subtitle</v>
+        <v>Plan Name</v>
       </c>
       <c r="D15" t="str">
-        <v>{{PAYMENT_FLEX_CANCEL_NOTICE}}</v>
+        <v>{{PAYMENT_PLAN_NAME}}</v>
       </c>
       <c r="E15" t="str">
         <v/>
@@ -4729,10 +4760,10 @@
         <v>Monthly</v>
       </c>
       <c r="C16" t="str">
-        <v>First Month Free Price</v>
+        <v>Plan Subtitle</v>
       </c>
       <c r="D16" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{PAYMENT_FLEX_CANCEL_NOTICE}}</v>
       </c>
       <c r="E16" t="str">
         <v/>
@@ -4746,10 +4777,10 @@
         <v>Monthly</v>
       </c>
       <c r="C17" t="str">
-        <v>First Month Free Text</v>
+        <v>First Month Free Price</v>
       </c>
       <c r="D17" t="str">
-        <v>{{PAYMENT_FREE_TEXT}}</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E17" t="str">
         <v/>
@@ -4763,10 +4794,10 @@
         <v>Monthly</v>
       </c>
       <c r="C18" t="str">
-        <v>PPV Name</v>
+        <v>First Month Free Text</v>
       </c>
       <c r="D18" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>{{PAYMENT_FREE_TEXT}}</v>
       </c>
       <c r="E18" t="str">
         <v/>
@@ -4780,10 +4811,10 @@
         <v>Monthly</v>
       </c>
       <c r="C19" t="str">
-        <v>PPV Price</v>
+        <v>PPV Name</v>
       </c>
       <c r="D19" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="E19" t="str">
         <v/>
@@ -4797,10 +4828,10 @@
         <v>Monthly</v>
       </c>
       <c r="C20" t="str">
-        <v>Today You Pay Text</v>
+        <v>PPV Price</v>
       </c>
       <c r="D20" t="str">
-        <v>Today you pay</v>
+        <v>{{PPV_PRICE}}</v>
       </c>
       <c r="E20" t="str">
         <v/>
@@ -4814,10 +4845,10 @@
         <v>Monthly</v>
       </c>
       <c r="C21" t="str">
-        <v>Today You Pay Price</v>
+        <v>Today You Pay Text</v>
       </c>
       <c r="D21" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>Today you pay</v>
       </c>
       <c r="E21" t="str">
         <v/>
@@ -4831,10 +4862,10 @@
         <v>Monthly</v>
       </c>
       <c r="C22" t="str">
-        <v>Cancellation Text</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D22" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>{{PPV_PRICE}}</v>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -4848,10 +4879,10 @@
         <v>Monthly</v>
       </c>
       <c r="C23" t="str">
-        <v>Legal Text</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D23" t="str">
-        <v>{{PAYMENT_FLEX_LEGAL_TEXT}}</v>
+        <v>{{CANCELLATION_TEXT}}</v>
       </c>
       <c r="E23" t="str">
         <v/>
@@ -4865,10 +4896,10 @@
         <v>Monthly</v>
       </c>
       <c r="C24" t="str">
-        <v>Ultimate Upsell Text</v>
+        <v>Legal Text</v>
       </c>
       <c r="D24" t="str">
-        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
+        <v>{{PAYMENT_FLEX_LEGAL_TEXT}}</v>
       </c>
       <c r="E24" t="str">
         <v/>
@@ -4879,13 +4910,13 @@
         <v>Standard</v>
       </c>
       <c r="B25" t="str">
-        <v>Annual Pay Monthly</v>
+        <v>Monthly</v>
       </c>
       <c r="C25" t="str">
-        <v>Page Title</v>
+        <v>Ultimate Upsell Text</v>
       </c>
       <c r="D25" t="str">
-        <v>Choose how to pay</v>
+        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
       <c r="E25" t="str">
         <v/>
@@ -4899,10 +4930,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C26" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D26" t="str">
-        <v>DAZN Standard</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E26" t="str">
         <v/>
@@ -4916,10 +4947,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C27" t="str">
-        <v>PPV Name</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D27" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>DAZN Standard</v>
       </c>
       <c r="E27" t="str">
         <v/>
@@ -4933,10 +4964,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C28" t="str">
-        <v>PPV Price</v>
+        <v>PPV Name</v>
       </c>
       <c r="D28" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="E28" t="str">
         <v/>
@@ -4950,10 +4981,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C29" t="str">
-        <v>Rate Plan</v>
+        <v>PPV Price</v>
       </c>
       <c r="D29" t="str">
-        <v>{{RATE_PLAN_LABEL}}</v>
+        <v>{{PPV_PRICE}}</v>
       </c>
       <c r="E29" t="str">
         <v/>
@@ -4967,10 +4998,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C30" t="str">
-        <v>Rate Plan Original Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D30" t="str">
-        <v>{{CURRENCY}}{{ANNUAL_PRICE}}</v>
+        <v>{{RATE_PLAN_LABEL}}</v>
       </c>
       <c r="E30" t="str">
         <v/>
@@ -4984,10 +5015,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C31" t="str">
-        <v>Rate Plan Discounted Price</v>
+        <v>Rate Plan Original Price</v>
       </c>
       <c r="D31" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{CURRENCY}}{{ANNUAL_PRICE}}</v>
       </c>
       <c r="E31" t="str">
         <v/>
@@ -5001,10 +5032,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C32" t="str">
-        <v>Today You Pay Text</v>
+        <v>Rate Plan Discounted Price</v>
       </c>
       <c r="D32" t="str">
-        <v>Today you pay</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E32" t="str">
         <v/>
@@ -5018,10 +5049,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C33" t="str">
-        <v>Today You Pay Price</v>
+        <v>Today You Pay Text</v>
       </c>
       <c r="D33" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>Today you pay</v>
       </c>
       <c r="E33" t="str">
         <v/>
@@ -5035,10 +5066,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C34" t="str">
-        <v>Cancellation Text</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D34" t="str">
-        <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
+        <v>{{PPV_PRICE}}</v>
       </c>
       <c r="E34" t="str">
         <v/>
@@ -5052,10 +5083,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C35" t="str">
-        <v>Redeem Promo Code CTA</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D35" t="str">
-        <v>Yes</v>
+        <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
       </c>
       <c r="E35" t="str">
         <v/>
@@ -5069,10 +5100,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C36" t="str">
-        <v>Ultimate Upsell Text</v>
+        <v>Redeem Promo Code CTA</v>
       </c>
       <c r="D36" t="str">
-        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
+        <v>Yes</v>
       </c>
       <c r="E36" t="str">
         <v/>
@@ -5080,16 +5111,16 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Ultimate</v>
+        <v>Standard</v>
       </c>
       <c r="B37" t="str">
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C37" t="str">
-        <v>Page Title</v>
+        <v>Ultimate Upsell Text</v>
       </c>
       <c r="D37" t="str">
-        <v>Choose how to pay</v>
+        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
       <c r="E37" t="str">
         <v/>
@@ -5103,10 +5134,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C38" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D38" t="str">
-        <v>DAZN Ultimate</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E38" t="str">
         <v/>
@@ -5120,10 +5151,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C39" t="str">
-        <v>PPV Name</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D39" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="E39" t="str">
         <v/>
@@ -5137,10 +5168,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C40" t="str">
-        <v>PPV Price</v>
+        <v>PPV Name</v>
       </c>
       <c r="D40" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="E40" t="str">
         <v/>
@@ -5154,10 +5185,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C41" t="str">
-        <v>Rate Plan</v>
+        <v>PPV Price</v>
       </c>
       <c r="D41" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E41" t="str">
         <v/>
@@ -5171,10 +5202,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C42" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D42" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
+        <v>Annual - Pay Monthly</v>
       </c>
       <c r="E42" t="str">
         <v/>
@@ -5188,10 +5219,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C43" t="str">
-        <v>Plan Subtitle</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="D43" t="str">
-        <v>Billed monthly. 12-month contract.</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
       <c r="E43" t="str">
         <v/>
@@ -5205,10 +5236,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C44" t="str">
-        <v>Today You Pay Text</v>
+        <v>Plan Subtitle</v>
       </c>
       <c r="D44" t="str">
-        <v>Today you pay</v>
+        <v>Billed monthly. 12-month contract.</v>
       </c>
       <c r="E44" t="str">
         <v/>
@@ -5222,10 +5253,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C45" t="str">
-        <v>Today You Pay Price</v>
+        <v>Today You Pay Text</v>
       </c>
       <c r="D45" t="str">
-        <v>{{TODAY_YOU_PAY_PRICE}}</v>
+        <v>Today you pay</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -5239,10 +5270,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C46" t="str">
-        <v>Next Payment Label</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D46" t="str">
-        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
       <c r="E46" t="str">
         <v/>
@@ -5256,10 +5287,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C47" t="str">
-        <v>Next Payment Price</v>
+        <v>Next Payment Label</v>
       </c>
       <c r="D47" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
+        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
       <c r="E47" t="str">
         <v/>
@@ -5273,10 +5304,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C48" t="str">
-        <v>Cancellation Text</v>
+        <v>Next Payment Price</v>
       </c>
       <c r="D48" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
       <c r="E48" t="str">
         <v/>
@@ -5290,10 +5321,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C49" t="str">
-        <v>Redeem Promo Code CTA</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D49" t="str">
-        <v>Yes</v>
+        <v>{{CANCELLATION_TEXT}}</v>
       </c>
       <c r="E49" t="str">
         <v/>
@@ -5307,10 +5338,10 @@
         <v>Annual Pay Monthly</v>
       </c>
       <c r="C50" t="str">
-        <v>Discount Badge</v>
+        <v>Redeem Promo Code CTA</v>
       </c>
       <c r="D50" t="str">
-        <v>{{DISCOUNT_BADGE}}</v>
+        <v>Yes</v>
       </c>
       <c r="E50" t="str">
         <v/>
@@ -5321,13 +5352,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B51" t="str">
-        <v>Annual Pay Upfront</v>
+        <v>Annual Pay Monthly</v>
       </c>
       <c r="C51" t="str">
-        <v>Page Title</v>
+        <v>Discount Badge</v>
       </c>
       <c r="D51" t="str">
-        <v>Choose how to pay</v>
+        <v>{{DISCOUNT_BADGE}}</v>
       </c>
       <c r="E51" t="str">
         <v/>
@@ -5341,10 +5372,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C52" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D52" t="str">
-        <v>DAZN Ultimate</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E52" t="str">
         <v/>
@@ -5358,10 +5389,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C53" t="str">
-        <v>PPV Name</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D53" t="str">
-        <v>{{PPV_NAME}}</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="E53" t="str">
         <v/>
@@ -5375,10 +5406,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C54" t="str">
-        <v>PPV Price</v>
+        <v>PPV Name</v>
       </c>
       <c r="D54" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{PPV_NAME}}</v>
       </c>
       <c r="E54" t="str">
         <v/>
@@ -5392,10 +5423,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C55" t="str">
-        <v>Rate Plan</v>
+        <v>PPV Price</v>
       </c>
       <c r="D55" t="str">
-        <v>Annual - Pay Upfront</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E55" t="str">
         <v/>
@@ -5409,10 +5440,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C56" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D56" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
+        <v>Annual - Pay Upfront</v>
       </c>
       <c r="E56" t="str">
         <v/>
@@ -5426,10 +5457,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C57" t="str">
-        <v>Plan Subtitle</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="D57" t="str">
-        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}. Pay for the full year up front!|Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
+        <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
       </c>
       <c r="E57" t="str">
         <v/>
@@ -5443,10 +5474,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C58" t="str">
-        <v>Today You Pay Text</v>
+        <v>Plan Subtitle</v>
       </c>
       <c r="D58" t="str">
-        <v>Today you pay</v>
+        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}. Pay for the full year up front|Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
       <c r="E58" t="str">
         <v/>
@@ -5460,10 +5491,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C59" t="str">
-        <v>Today You Pay Price</v>
+        <v>Today You Pay Text</v>
       </c>
       <c r="D59" t="str">
-        <v>{{TODAY_YOU_PAY_PRICE}}</v>
+        <v>Today you pay</v>
       </c>
       <c r="E59" t="str">
         <v/>
@@ -5477,10 +5508,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C60" t="str">
-        <v>Next Payment Label</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D60" t="str">
-        <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
       <c r="E60" t="str">
         <v/>
@@ -5494,10 +5525,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C61" t="str">
-        <v>Next Payment Price</v>
+        <v>Next Payment Label</v>
       </c>
       <c r="D61" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
+        <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
       <c r="E61" t="str">
         <v/>
@@ -5511,10 +5542,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C62" t="str">
-        <v>Cancellation Text</v>
+        <v>Next Payment Price</v>
       </c>
       <c r="D62" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
       <c r="E62" t="str">
         <v/>
@@ -5528,10 +5559,10 @@
         <v>Annual Pay Upfront</v>
       </c>
       <c r="C63" t="str">
-        <v>Redeem Promo Code CTA</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D63" t="str">
-        <v>Yes</v>
+        <v>{{CANCELLATION_TEXT}}</v>
       </c>
       <c r="E63" t="str">
         <v/>
@@ -5539,16 +5570,16 @@
     </row>
     <row r="64">
       <c r="A64" t="str">
-        <v>Standard</v>
+        <v>Ultimate</v>
       </c>
       <c r="B64" t="str">
-        <v>Monthly Bundle</v>
+        <v>Annual Pay Upfront</v>
       </c>
       <c r="C64" t="str">
-        <v>Page Title</v>
+        <v>Redeem Promo Code CTA</v>
       </c>
       <c r="D64" t="str">
-        <v>{{PAYMENT_PAGE_TITLE}}</v>
+        <v>Yes</v>
       </c>
       <c r="E64" t="str">
         <v/>
@@ -5562,10 +5593,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C65" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D65" t="str">
-        <v>DAZN Standard</v>
+        <v>{{PAYMENT_PAGE_TITLE}}</v>
       </c>
       <c r="E65" t="str">
         <v/>
@@ -5579,10 +5610,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C66" t="str">
-        <v>Bundle Name</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D66" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>DAZN Standard</v>
       </c>
       <c r="E66" t="str">
         <v/>
@@ -5596,10 +5627,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C67" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Name</v>
       </c>
       <c r="D67" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="E67" t="str">
         <v/>
@@ -5613,10 +5644,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C68" t="str">
-        <v>Today You Pay Price</v>
+        <v>Bundle Price</v>
       </c>
       <c r="D68" t="str">
-        <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="E68" t="str">
         <v/>
@@ -5630,10 +5661,10 @@
         <v>Monthly Bundle</v>
       </c>
       <c r="C69" t="str">
-        <v>Cancellation Text</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D69" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
       </c>
       <c r="E69" t="str">
         <v/>
@@ -5644,13 +5675,13 @@
         <v>Standard</v>
       </c>
       <c r="B70" t="str">
-        <v>Annual Pay Monthly Bundle</v>
+        <v>Monthly Bundle</v>
       </c>
       <c r="C70" t="str">
-        <v>Page Title</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D70" t="str">
-        <v>Choose how to pay</v>
+        <v>{{CANCELLATION_TEXT}}</v>
       </c>
       <c r="E70" t="str">
         <v/>
@@ -5664,10 +5695,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C71" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D71" t="str">
-        <v>DAZN Standard</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E71" t="str">
         <v/>
@@ -5681,10 +5712,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C72" t="str">
-        <v>Rate Plan</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D72" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>DAZN Standard</v>
       </c>
       <c r="E72" t="str">
         <v/>
@@ -5698,10 +5729,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C73" t="str">
-        <v>First Month Free Text</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D73" t="str">
-        <v>First month free</v>
+        <v>Annual - Pay Monthly</v>
       </c>
       <c r="E73" t="str">
         <v/>
@@ -5715,10 +5746,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C74" t="str">
-        <v>Bundle Name</v>
+        <v>First Month Free Text</v>
       </c>
       <c r="D74" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>First month free</v>
       </c>
       <c r="E74" t="str">
         <v/>
@@ -5732,10 +5763,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C75" t="str">
-        <v>Bundle Original Price</v>
+        <v>Bundle Name</v>
       </c>
       <c r="D75" t="str">
-        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="E75" t="str">
         <v/>
@@ -5749,10 +5780,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C76" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Original Price</v>
       </c>
       <c r="D76" t="str">
-        <v>{{BUNDLE_PRICE}}</v>
+        <v>{{BUNDLE_ORIGINAL_PRICE}}</v>
       </c>
       <c r="E76" t="str">
         <v/>
@@ -5766,10 +5797,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C77" t="str">
-        <v>Bundle Discount</v>
+        <v>Bundle Price</v>
       </c>
       <c r="D77" t="str">
-        <v>{{BUNDLE_DISCOUNT}}</v>
+        <v>{{BUNDLE_PRICE}}</v>
       </c>
       <c r="E77" t="str">
         <v/>
@@ -5783,10 +5814,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C78" t="str">
-        <v>Today You Pay Price</v>
+        <v>Bundle Discount</v>
       </c>
       <c r="D78" t="str">
-        <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
+        <v>{{BUNDLE_DISCOUNT}}</v>
       </c>
       <c r="E78" t="str">
         <v/>
@@ -5800,10 +5831,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C79" t="str">
-        <v>Cancellation Text</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D79" t="str">
-        <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
+        <v>{{BUNDLE_TODAY_YOU_PAY_STANDARD}}</v>
       </c>
       <c r="E79" t="str">
         <v/>
@@ -5817,10 +5848,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C80" t="str">
-        <v>Ultimate Upsell Text</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D80" t="str">
-        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
+        <v>{{CANCELLATION_TEXT_ANNUAL}}</v>
       </c>
       <c r="E80" t="str">
         <v/>
@@ -5828,16 +5859,16 @@
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Ultimate</v>
+        <v>Standard</v>
       </c>
       <c r="B81" t="str">
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C81" t="str">
-        <v>Page Title</v>
+        <v>Ultimate Upsell Text</v>
       </c>
       <c r="D81" t="str">
-        <v>Choose how to pay</v>
+        <v>Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost – {{UPSELL_PRICE}}/month|Switch to DAZN Ultimate and enjoy pay-per-views at no extra cost|N/A</v>
       </c>
       <c r="E81" t="str">
         <v/>
@@ -5851,10 +5882,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C82" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D82" t="str">
-        <v>DAZN Ultimate</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E82" t="str">
         <v/>
@@ -5868,10 +5899,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C83" t="str">
-        <v>Rate Plan</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D83" t="str">
-        <v>Annual - Pay Monthly</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="E83" t="str">
         <v/>
@@ -5885,10 +5916,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C84" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D84" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
+        <v>Annual - Pay Monthly</v>
       </c>
       <c r="E84" t="str">
         <v/>
@@ -5902,10 +5933,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C85" t="str">
-        <v>Bundle Name</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="D85" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}/month</v>
       </c>
       <c r="E85" t="str">
         <v/>
@@ -5919,10 +5950,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C86" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Name</v>
       </c>
       <c r="D86" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="E86" t="str">
         <v/>
@@ -5936,10 +5967,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C87" t="str">
-        <v>Today You Pay Price</v>
+        <v>Bundle Price</v>
       </c>
       <c r="D87" t="str">
-        <v>{{TODAY_YOU_PAY_PRICE}}</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E87" t="str">
         <v/>
@@ -5953,10 +5984,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C88" t="str">
-        <v>Next Payment Label</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D88" t="str">
-        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
       <c r="E88" t="str">
         <v/>
@@ -5970,10 +6001,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C89" t="str">
-        <v>Next Payment Price</v>
+        <v>Next Payment Label</v>
       </c>
       <c r="D89" t="str">
-        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
+        <v>Next payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
       <c r="E89" t="str">
         <v/>
@@ -5987,10 +6018,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C90" t="str">
-        <v>Cancellation Text</v>
+        <v>Next Payment Price</v>
       </c>
       <c r="D90" t="str">
-        <v>{{CANCELLATION_TEXT}}</v>
+        <v>{{ANNUAL_PAY_MONTHLY_PRICE}}</v>
       </c>
       <c r="E90" t="str">
         <v/>
@@ -6004,10 +6035,10 @@
         <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C91" t="str">
-        <v>Discount Badge</v>
+        <v>Cancellation Text</v>
       </c>
       <c r="D91" t="str">
-        <v>{{DISCOUNT_BADGE}}</v>
+        <v>{{CANCELLATION_TEXT}}</v>
       </c>
       <c r="E91" t="str">
         <v/>
@@ -6018,13 +6049,13 @@
         <v>Ultimate</v>
       </c>
       <c r="B92" t="str">
-        <v>Annual Pay Upfront Bundle</v>
+        <v>Annual Pay Monthly Bundle</v>
       </c>
       <c r="C92" t="str">
-        <v>Page Title</v>
+        <v>Discount Badge</v>
       </c>
       <c r="D92" t="str">
-        <v>Choose how to pay</v>
+        <v>{{DISCOUNT_BADGE}}</v>
       </c>
       <c r="E92" t="str">
         <v/>
@@ -6038,10 +6069,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C93" t="str">
-        <v>DAZN Tier</v>
+        <v>Page Title</v>
       </c>
       <c r="D93" t="str">
-        <v>DAZN Ultimate</v>
+        <v>Choose how to pay</v>
       </c>
       <c r="E93" t="str">
         <v/>
@@ -6055,10 +6086,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C94" t="str">
-        <v>Rate Plan</v>
+        <v>DAZN Tier</v>
       </c>
       <c r="D94" t="str">
-        <v>Annual - Pay Upfront</v>
+        <v>DAZN Ultimate</v>
       </c>
       <c r="E94" t="str">
         <v/>
@@ -6072,10 +6103,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C95" t="str">
-        <v>Rate Plan Price</v>
+        <v>Rate Plan</v>
       </c>
       <c r="D95" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
+        <v>Annual - Pay Upfront</v>
       </c>
       <c r="E95" t="str">
         <v/>
@@ -6089,10 +6120,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C96" t="str">
-        <v>Save Badge</v>
+        <v>Rate Plan Price</v>
       </c>
       <c r="D96" t="str">
-        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
+        <v>{{ANNUAL_UPFRONT_PRICE}}/year</v>
       </c>
       <c r="E96" t="str">
         <v/>
@@ -6106,10 +6137,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C97" t="str">
-        <v>Bundle Name</v>
+        <v>Save Badge</v>
       </c>
       <c r="D97" t="str">
-        <v>{{BUNDLE_NAME}}</v>
+        <v>Save {{CURRENCY}}{{UPFRONT_SAVE_AMOUNT}}</v>
       </c>
       <c r="E97" t="str">
         <v/>
@@ -6123,10 +6154,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C98" t="str">
-        <v>Bundle Price</v>
+        <v>Bundle Name</v>
       </c>
       <c r="D98" t="str">
-        <v>{{CURRENCY}}0</v>
+        <v>{{BUNDLE_NAME}}</v>
       </c>
       <c r="E98" t="str">
         <v/>
@@ -6140,10 +6171,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C99" t="str">
-        <v>Today You Pay Price</v>
+        <v>Bundle Price</v>
       </c>
       <c r="D99" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
+        <v>{{CURRENCY}}0</v>
       </c>
       <c r="E99" t="str">
         <v/>
@@ -6157,10 +6188,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C100" t="str">
-        <v>Next Payment Label</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="D100" t="str">
-        <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
+        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
       </c>
       <c r="E100" t="str">
         <v/>
@@ -6174,10 +6205,10 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C101" t="str">
-        <v>Next Payment Price</v>
+        <v>Next Payment Label</v>
       </c>
       <c r="D101" t="str">
-        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
+        <v>Next Annual payment on {{NEXT_PAYMENT_DATE}}</v>
       </c>
       <c r="E101" t="str">
         <v/>
@@ -6191,18 +6222,35 @@
         <v>Annual Pay Upfront Bundle</v>
       </c>
       <c r="C102" t="str">
+        <v>Next Payment Price</v>
+      </c>
+      <c r="D102" t="str">
+        <v>{{ANNUAL_UPFRONT_PRICE}}</v>
+      </c>
+      <c r="E102" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="str">
+        <v>Ultimate</v>
+      </c>
+      <c r="B103" t="str">
+        <v>Annual Pay Upfront Bundle</v>
+      </c>
+      <c r="C103" t="str">
         <v>Cancellation Text</v>
       </c>
-      <c r="D102" t="str">
+      <c r="D103" t="str">
         <v>{{CANCELLATION_TEXT}}</v>
       </c>
-      <c r="E102" t="str">
+      <c r="E103" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E102"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E103"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6212,7 +6260,7 @@
   <dimension ref="A1:B15"/>
   <cols>
     <col min="1" max="1" width="27.83203125" customWidth="1"/>
-    <col min="2" max="2" width="21.83203125" customWidth="1"/>
+    <col min="2" max="2" width="90.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6308,7 +6356,7 @@
         <v>Popup Description</v>
       </c>
       <c r="B12" t="str">
-        <v>{{PPV_DESCRIPTION}}</v>
+        <v>Catch the biggest moment of the year. Select a DAZN plan to pair with your pay-per-view.</v>
       </c>
     </row>
     <row r="13">
@@ -6344,7 +6392,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
@@ -6414,9 +6462,17 @@
         <v>{{PPV_STATUS}}</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>PPV Image Present</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6622,10 +6678,10 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B18"/>
   <cols>
     <col min="1" max="1" width="29.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="79.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6756,9 +6812,25 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Payment Type</v>
+      </c>
+      <c r="B17" t="str">
+        <v>One time payment</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Payment Instruction Text</v>
+      </c>
+      <c r="B18" t="str">
+        <v>In order to purchase this event, please choose from the payment options below</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(android): add home-page-dont-miss and home-boxing-tile automation flow with title checking and visual validations
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -3770,7 +3770,7 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3860,10 +3860,75 @@
         <v>home-page-banner</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>PPV Tile Present</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C9" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>PPV Title</v>
+      </c>
+      <c r="B10" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+      <c r="C10" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>PPV Image Present</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C11" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Lock Icon</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C12" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Bell Icon</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C13" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>PPV Date</v>
+      </c>
+      <c r="B14" t="str">
+        <v>{{MOBILE_BANNER_MONTH}} {{MOBILE_SCHEDULE_DATE}}</v>
+      </c>
+      <c r="C14" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(excel): add PPV Tile validation fields for home-boxing-tile flow in Andriod_Home_Boxing_Page sheet
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -3935,7 +3935,7 @@
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4091,10 +4091,75 @@
         <v>home-boxing-upcoming</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>PPV Tile Present</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C15" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>PPV Title</v>
+      </c>
+      <c r="B16" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+      <c r="C16" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>PPV Image Present</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C17" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Lock Icon</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C18" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Bell Icon</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C19" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>PPV Date</v>
+      </c>
+      <c r="B20" t="str">
+        <v>{{MOBILE_BANNER_MONTH}} {{MOBILE_SCHEDULE_DATE}}</v>
+      </c>
+      <c r="C20" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C20"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(android): add home-page-dont-miss, home-boxing-tile flows, clear app data fix, and fixture validations across all tile flows
</commit_message>
<xml_diff>
--- a/data/PPV_Input.xlsx
+++ b/data/PPV_Input.xlsx
@@ -2200,7 +2200,7 @@
         <v>Page Heading</v>
       </c>
       <c r="B3" t="str">
-        <v>Buy {{PPV_NAME}} with a {{FREE_TRIAL_DAYS}}-day free trial</v>
+        <v>Buy {{PPV_NAME}} with a 7-day free trial</v>
       </c>
       <c r="C3" t="str">
         <v>checked</v>
@@ -2288,7 +2288,7 @@
         <v>Flex Badge</v>
       </c>
       <c r="B11" t="str">
-        <v>{{FLEX_BADGE}}</v>
+        <v>7 DAY FREE TRIAL</v>
       </c>
       <c r="C11" t="str">
         <v>checked</v>
@@ -2310,7 +2310,7 @@
         <v>Flex Today Text</v>
       </c>
       <c r="B13" t="str">
-        <v>{{FLEX_TODAY_TEXT}}</v>
+        <v>Only pay for the fight and start your 7-day free trial of DAZN Standard</v>
       </c>
       <c r="C13" t="str">
         <v>checked</v>
@@ -2321,7 +2321,7 @@
         <v>Flex Future Date</v>
       </c>
       <c r="B14" t="str">
-        <v>{{FLEX_FUTURE_DATE}}</v>
+        <v>In 7 days • {{FLEX_FUTURE_DATE_SHORT}}</v>
       </c>
       <c r="C14" t="str">
         <v>checked</v>
@@ -2387,7 +2387,7 @@
         <v>CTA Button (Flex selected)</v>
       </c>
       <c r="B20" t="str">
-        <v>{{PLAN_CTA_BUTTON_STANDARD}}</v>
+        <v>Continue with 7-day free trial</v>
       </c>
       <c r="C20" t="str">
         <v>checked</v>
@@ -3770,7 +3770,7 @@
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3860,17 +3860,82 @@
         <v>home-page-banner</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>PPV Tile Present</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C9" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>PPV Title</v>
+      </c>
+      <c r="B10" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+      <c r="C10" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>PPV Image Present</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C11" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Lock Icon</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C12" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Bell Icon</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C13" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>PPV Date</v>
+      </c>
+      <c r="B14" t="str">
+        <v>{{MOBILE_BANNER_MONTH}} {{MOBILE_SCHEDULE_DATE}}</v>
+      </c>
+      <c r="C14" t="str">
+        <v>home-page-dont-miss</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4026,10 +4091,75 @@
         <v>home-boxing-upcoming</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>PPV Tile Present</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C15" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>PPV Title</v>
+      </c>
+      <c r="B16" t="str">
+        <v>{{PPV_NAME}}</v>
+      </c>
+      <c r="C16" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>PPV Image Present</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C17" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Lock Icon</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C18" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Bell Icon</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="C19" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>PPV Date</v>
+      </c>
+      <c r="B20" t="str">
+        <v>{{MOBILE_BANNER_MONTH}} {{MOBILE_SCHEDULE_DATE}}</v>
+      </c>
+      <c r="C20" t="str">
+        <v>home-boxing-tile</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C20"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5232,7 +5362,7 @@
         <v>Trial Title</v>
       </c>
       <c r="C68" t="str">
-        <v>{{FREE_TRIAL_DAYS}}-day free trial of DAZN Standard</v>
+        <v>7-day free trial of DAZN Standard</v>
       </c>
     </row>
     <row r="69">
@@ -5265,7 +5395,7 @@
         <v>Trial Feature 1</v>
       </c>
       <c r="C71" t="str">
-        <v>{{FREE_TRIAL_DAYS}}-days free access to DAZN Standard.</v>
+        <v>7-days free access to DAZN Standard.</v>
       </c>
     </row>
     <row r="72">
@@ -5507,7 +5637,7 @@
         <v>CTA Button</v>
       </c>
       <c r="C93" t="str">
-        <v>Continue with PPV</v>
+        <v>Continue with PPV + 7-day free trial</v>
       </c>
     </row>
     <row r="94">
@@ -7932,7 +8062,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B18"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7963,7 +8093,7 @@
         <v>PPV Description</v>
       </c>
       <c r="B4" t="str">
-        <v>{{BANNER_DESCRIPTION}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="5">
@@ -7992,31 +8122,31 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Order Summary PPV Price</v>
+        <v>Today You Pay Text</v>
       </c>
       <c r="B8" t="str">
-        <v>{{PPV_PRICE}}</v>
+        <v>Today you pay</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Today You Pay Text</v>
+        <v>Today You Pay Price</v>
       </c>
       <c r="B9" t="str">
-        <v>Today you pay</v>
+        <v>{{TODAY_YOU_PAY_PRICE}}</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Today You Pay Price</v>
+        <v>Payment Method Present</v>
       </c>
       <c r="B10" t="str">
-        <v>{{TODAY_YOU_PAY_PRICE}}</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Payment Method Present</v>
+        <v>Pay Now Button</v>
       </c>
       <c r="B11" t="str">
         <v>Yes</v>
@@ -8024,7 +8154,7 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Pay Now Button</v>
+        <v>Secure Checkout</v>
       </c>
       <c r="B12" t="str">
         <v>Yes</v>
@@ -8032,7 +8162,7 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Secure Checkout</v>
+        <v>More Payment Methods</v>
       </c>
       <c r="B13" t="str">
         <v>Yes</v>
@@ -8040,7 +8170,7 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>More Payment Methods</v>
+        <v>Legal Text Present</v>
       </c>
       <c r="B14" t="str">
         <v>Yes</v>
@@ -8048,7 +8178,7 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Legal Text Present</v>
+        <v>Terms Link Present</v>
       </c>
       <c r="B15" t="str">
         <v>Yes</v>
@@ -8056,7 +8186,7 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Terms Link Present</v>
+        <v>Privacy Policy Link Present</v>
       </c>
       <c r="B16" t="str">
         <v>Yes</v>
@@ -8064,31 +8194,23 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Privacy Policy Link Present</v>
+        <v>Payment Type</v>
       </c>
       <c r="B17" t="str">
-        <v>Yes</v>
+        <v>One time payment</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Payment Type</v>
+        <v>Payment Instruction Text</v>
       </c>
       <c r="B18" t="str">
-        <v>One time payment</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Payment Instruction Text</v>
-      </c>
-      <c r="B19" t="str">
         <v>In order to purchase this event, please choose from the payment options below</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>